<commit_message>
Address transfers to a partner licensee, and fix a seeder import
A transfer template addressed to our own license technically passes but does
not demonstrate much. The counterparty is now configurable, so templates can
ship to a licensee in another sandbox tenant, and the transfer type follows
from that: unaffiliated when the recipient is outside our tenant, affiliated
within it.

Also fixes seed_inventory, which called _names without importing it — the
failure only showed when a facility needed seeding and had no strains.

Adds the drafted note to api-info@metrc.com covering the two endpoints that
return 401 on both tenants and the packages/adjust semantics.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WckmkszE5f38nyn3gphdpj
</commit_message>
<xml_diff>
--- a/evidence/metrc/Evaluation_NY_completed.xlsx
+++ b/evidence/metrc/Evaluation_NY_completed.xlsx
@@ -11145,12 +11145,12 @@
       </c>
       <c r="D5" s="248" t="inlineStr">
         <is>
-          <t>16006</t>
+          <t>15910</t>
         </is>
       </c>
       <c r="E5" s="250" t="inlineStr">
         <is>
-          <t>2026-08-27T14:02:18Z</t>
+          <t>2026-08-29T13:32:25Z</t>
         </is>
       </c>
       <c r="F5" s="247" t="inlineStr">
@@ -11165,7 +11165,7 @@
       </c>
       <c r="H5" s="262" t="inlineStr">
         <is>
-          <t>[{"Name":"TP Template A 0827-1402","TransporterFacilityLicenseNumber":null,"DriverOccupationalLicenseNumber":null,"DriverName":null,"DriverLicenseNumber":null,"PhoneNumberForQuestions":null,"VehicleMake":null,"VehicleModel":null,"VehicleLicensePlateNumber":null,"VehicleRegistrationNumber":null,"Destinations":[{"RecipientLicenseNumber":"SF-SBX-NY-5-30301","InvoiceNumber":"INV-A-0827-1402","TransferTypeName":"Affiliated Transfer","PlannedRoute":"Evaluation route.","EstimatedDepartureDateTime":"2026-08-27T15:02:16Z","EstimatedArrivalDateTime":"2026-08-27T18:02:16Z","Transporters":[],"Packages":[]}]}]</t>
+          <t>[{"Name":"TP Template A 0829-1332","TransporterFacilityLicenseNumber":null,"DriverOccupationalLicenseNumber":null,"DriverName":null,"DriverLicenseNumber":null,"PhoneNumberForQuestions":null,"VehicleMake":null,"VehicleModel":null,"VehicleLicensePlateNumber":null,"VehicleRegistrationNumber":null,"Destinations":[{"RecipientLicenseNumber":"SF-SBX-NY-6-13402","InvoiceNumber":"INV-A-0829-1332","TransferTypeName":"Unaffiliated Transfer","PlannedRoute":"Evaluation route.","EstimatedDepartureDateTime":"2026-08-29T14:32:24Z","EstimatedArrivalDateTime":"2026-08-29T17:32:24Z","Transporters":[],"Packages":[]}]}]</t>
         </is>
       </c>
     </row>
@@ -11219,12 +11219,12 @@
       </c>
       <c r="D9" s="248" t="inlineStr">
         <is>
-          <t>16007</t>
+          <t>15911</t>
         </is>
       </c>
       <c r="E9" s="250" t="inlineStr">
         <is>
-          <t>2026-08-27T14:02:18Z</t>
+          <t>2026-08-29T13:32:25Z</t>
         </is>
       </c>
       <c r="F9" s="247" t="inlineStr">
@@ -11239,7 +11239,7 @@
       </c>
       <c r="H9" s="262" t="inlineStr">
         <is>
-          <t>[{"Name":"TP Template B 0827-1402","TransporterFacilityLicenseNumber":null,"DriverOccupationalLicenseNumber":null,"DriverName":null,"DriverLicenseNumber":null,"PhoneNumberForQuestions":null,"VehicleMake":null,"VehicleModel":null,"VehicleLicensePlateNumber":null,"VehicleRegistrationNumber":null,"Destinations":[{"RecipientLicenseNumber":"SF-SBX-NY-5-30301","InvoiceNumber":"INV-B-0827-1402","TransferTypeName":"Affiliated Transfer","PlannedRoute":"Evaluation route.","EstimatedDepartureDateTime":"2026-08-27T15:02:16Z","EstimatedArrivalDateTime":"2026-08-27T18:02:16Z","Transporters":[],"Packages":[]}]}]</t>
+          <t>[{"Name":"TP Template B 0829-1332","TransporterFacilityLicenseNumber":null,"DriverOccupationalLicenseNumber":null,"DriverName":null,"DriverLicenseNumber":null,"PhoneNumberForQuestions":null,"VehicleMake":null,"VehicleModel":null,"VehicleLicensePlateNumber":null,"VehicleRegistrationNumber":null,"Destinations":[{"RecipientLicenseNumber":"SF-SBX-NY-6-13402","InvoiceNumber":"INV-B-0829-1332","TransferTypeName":"Unaffiliated Transfer","PlannedRoute":"Evaluation route.","EstimatedDepartureDateTime":"2026-08-29T14:32:24Z","EstimatedArrivalDateTime":"2026-08-29T17:32:24Z","Transporters":[],"Packages":[]}]}]</t>
         </is>
       </c>
     </row>
@@ -11292,12 +11292,12 @@
       </c>
       <c r="D13" s="248" t="inlineStr">
         <is>
-          <t>16006, 16007</t>
+          <t>15910, 15911</t>
         </is>
       </c>
       <c r="E13" s="250" t="inlineStr">
         <is>
-          <t>2026-08-27T14:02:18+00:00</t>
+          <t>2026-08-29T13:32:25+00:00</t>
         </is>
       </c>
       <c r="F13" s="247" t="inlineStr">
@@ -11307,12 +11307,12 @@
       </c>
       <c r="G13" s="247" t="inlineStr">
         <is>
-          <t>https://sandbox-api-ny.metrc.com/transfers/v2/templates/outgoing?lastModifiedStart=2026-08-26T14%3A02%3A18Z&amp;lastModifiedEnd=2026-08-27T14%3A02%3A18Z&amp;licenseNumber=SF-SBX-NY-3-30301</t>
+          <t>https://sandbox-api-ny.metrc.com/transfers/v2/templates/outgoing?lastModifiedStart=2026-08-28T13%3A32%3A25Z&amp;lastModifiedEnd=2026-08-29T13%3A32%3A25Z&amp;licenseNumber=SF-SBX-NY-3-30301</t>
         </is>
       </c>
       <c r="H13" s="262" t="inlineStr">
         <is>
-          <t>{"Data":[{"Id":16006,"ManifestNumber":"T-0000016006","InvoiceNumber":"INV-A-0827-1402","ShipmentLicenseType":"Licensed","ShipperFacilityLicenseNumber":"SF-SBX-NY-3-30301","ShipperFacilityName":"Sandbox AU Cultivator","Name":"TP Template A 0827-1402","TransporterFacilityLicenseNumber":null,"TransporterFacilityName":null,"DriverName":null,"DriverOccupationalLicenseNumber":null,"DriverVehicleLicenseNumber":null,"VehicleMake":null,"VehicleModel":null,"VehicleLicensePlateNumber":null,"VehicleRegistrationNumber":null,"DeliveryCount":1,"ReceivedDeliveryCount":0,"PackageCount":0,"ReceivedPackageCount":0,"ContainsPlantPackage":false,"ContainsProductPackage":false,"ContainsTradeSample":false,"ContainsDonation":false,"ContainsTestingSample":false,"ContainsProductRequiresRemediation":false,"ContainsRemediatedProductPackage":false,"ContainsPreTreatedProductPackage":false,"IsVoided":false,"CreatedDateTime":"2026-08-27T14:02:18+00:00","CreatedByUserName":"Pablo Dayton","LastModified":"2026-08-27T14:02:18+00:00","DeliveryId":0,"RecipientFacilityLicenseNumber":null,"RecipientFacilityName":null,"ShipmentTypeName":null,"ShipmentTransactionType":null,"EstimatedDepartureDateTime":"0001-01-01T00:00:00.000","ActualDepartureDateTime":null,"EstimatedArrivalDateTime":"0001-01-01T00:00:00.000","ActualArrivalDateTime":null,"DeliveryPackageCount":0,"DeliveryReceivedPackageCount":0,"ReceivedDateTime":null,"EstimatedReturnDepartureDateTime":null,"ActualReturnDepartureDateTime":null,"EstimatedReturnArrivalDateTime":null,"ActualReturnArrivalDateTime":null,"OriginatingTemplateId":null},{"Id":16007,"ManifestNumber":"T-0000016007","InvoiceNumber":"INV-B-0827-1402","ShipmentLicenseType":"Licensed","ShipperFacilityLicenseNumber":"SF-SBX-NY-3-30301","ShipperFacilityName":"Sandbox AU Cultivator","Name":"TP Template B 0827-1402","TransporterFacilityLicenseNumber":null,"TransporterFacilityName":null,"DriverName":null,"DriverOccupationalLicenseNumber":null,"DriverVehicleLicenseNumber":null,"VehicleMake":null,"VehicleModel":null,"VehicleLicensePlateNumber":null,"VehicleRegistrationNumber":null,"DeliveryCount":1,"ReceivedDeliveryCount":0,"PackageCount":0,"ReceivedPackageCount":0,"ContainsPlantPackage":false,"ContainsProductPackage":false,"ContainsTradeSample":false,"ContainsDonation":false,"ContainsTestingSample":false,"ContainsProductRequiresRemediation":false,"ContainsRemediatedProductPackage":false,"ContainsPreTreatedProductPackage":false,"IsVoided":false,"CreatedDateTime":"2026-08-27T14:02:18+00:00","CreatedByUserName":"Pablo Dayton","LastModified":"2026-08-27T14:02:18+00:00","DeliveryId":0,"RecipientFacilityLicenseNumber":null,"RecipientFacilityName":null,"ShipmentTypeName":null,"ShipmentTransactionType":null,"EstimatedDepartureDateTime":"0001-01-01T00:00:00.000","ActualDepartureDateTime":null,"EstimatedArrivalDateTime":"0001-01-01T00:00:00.000","ActualArrivalDateTime":null,"DeliveryPackageCount":0,"DeliveryReceivedPackageCount":0,"ReceivedDateTime":null,"EstimatedReturnDepartureDateTime":null,"ActualReturnDepartureDateTime":null,"EstimatedReturnArrivalDateTime":null,"ActualReturnArrivalDateTime":null,"OriginatingTemplateId":null},{"Id":15909,"ManifestNumber":"T-0000015909","InvoiceNumber":"INV-A-0827-1400","ShipmentLicenseType":"Licensed","ShipperFacilityLicenseNumber":"SF-SBX-NY-3-30301","ShipperFacilityName":"Sandbox AU Cultivator","Name":"TP Template A 0827-1400 (Updated)","TransporterFacilityLicenseNumber":null,"TransporterFacilityName":null,"DriverName":null,"DriverOccupationalLicenseNumber":null,"DriverVehicleLicenseNumber":null,"VehicleMake":null,"VehicleModel":null,"VehicleLicensePlateNumber":null,"VehicleRegistrationNumber":null,"DeliveryCount":1,"ReceivedDeliveryCount":0,"PackageCount":0,"ReceivedPackageCount":0,"ContainsPlantPackage":false,"ContainsProductPackage":false,"ContainsTradeSample":false,"ContainsDonation":false,"ContainsTestingSample":false,"ContainsProductRequiresRemediation":false,"ContainsRemediatedProductPackage":false,"ContainsPreTreatedProductPackage":false,"IsVoided":false,"CreatedDateTime":"2026-08-27T14:00:28+00:00","CreatedByUserName":"Pablo Dayton","LastModified":"2026-08-27T14:00:28+00:00","DeliveryId":0,"RecipientFacilityLicenseNumber":null,"RecipientFacilityName":null,"ShipmentTypeName":null,"ShipmentTransactionType":null,"EstimatedDepartureDateTime":"0001-01-01T00:00:00.000","ActualDepartureDateTime":null,"EstimatedArrivalDateTime":"0001-01-01T00:00:00.000","ActualArrivalDateTime":null,"DeliveryPackageCount":0,"DeliveryReceivedPackageCount":0,"ReceivedDateTime":null,"EstimatedReturnDepartureDateTime":null,"ActualReturnDepartureDateTime":null,"EstimatedReturnArrivalDateTime":null,"ActualReturnArrivalDateTime":null,"OriginatingTemplateId":null},{"Id":16005,"ManifestNumber":"T-0000016005","InvoiceNumber":"INV-B-0827-1400","ShipmentLicenseType":"Licensed","ShipperFacilityLicenseNumber":"SF-SBX-NY-3-30301","ShipperFacilityName":"Sandbox AU Cultivator","Name":"TP Template B 0827-1400","TransporterFacilityLicenseNumber":null,"TransporterFacilityName":null,"DriverName":null,"DriverOccupationalLicenseNumber":null,"DriverVehicleLicenseNumber":null,"VehicleMake":null,"VehicleModel":null,"VehicleLicensePlateNumber":null,"VehicleRegistrationNumber":null,"DeliveryCount":1,"ReceivedDeliveryCount":0,"PackageCount":0,"ReceivedPackageCount":0,"ContainsPlantPackage":false,"ContainsProductPackage":false,"ContainsTradeSample":false,"ContainsDonation":false,"ContainsTestingSample":false,"ContainsProductRequiresRemediation":false,"ContainsRemediatedProductPackage":false,"ContainsPreTreatedProductPackage":false,"IsVoided":false,"CreatedDateTime":"2026-08-27T14:00:28+00:00","CreatedByUserName":"Pablo Dayton","LastModified":"2026-08-27T14:00:28+00:00","DeliveryId":0,"RecipientFacilityLicenseNumber":null,"RecipientFacilityName":null,"ShipmentTypeName":null,"ShipmentTransactionType":null,"EstimatedDepartureDateTime":"0001-01-01T00:00:00.000","ActualDepartureDateTime":null,"EstimatedArrivalDateTime":"0001-01-01T00:00:00.000","ActualArrivalDateTime":null,"DeliveryPackageCount":0,"DeliveryReceivedPackageCount":0,"ReceivedDateTime":null,"EstimatedReturnDepartureDateTime":null,"ActualReturnDepartureDateTime":null,"EstimatedReturnArrivalDateTime":null,"ActualReturnArrivalDateTime":null,"OriginatingTemplateId":null},{"Id":15907,"ManifestNumber":"T-0000015907","InvoiceNumber":"INV-A-0827-1359","ShipmentLicenseType":"Licensed","ShipperFacilityLicenseNumber":"SF-SBX-NY-3-30301","ShipperFacilityName":"Sandbox AU Cultivator","Name":"TP Template A 0827-1359 (Updated)","TransporterFacilityLicenseNumber":null,"TransporterFacilityName":null,"DriverName":null,"DriverOccupationalLicenseNumber":null,"DriverVehicleLicenseNumber":null,"VehicleMake":null,"VehicleModel":null,"VehicleLicensePlateNumber":null,"VehicleRegistrationNumber":null,"DeliveryCount":1,"ReceivedDeliveryCount":0,"PackageCount":0,"ReceivedPackageCount":0,"ContainsPlantPackage":false,"ContainsProductPackage":false,"ContainsTradeSample":false,"ContainsDonation":false,"ContainsTestingSample":false,"ContainsProductRequiresRemediation":false,"ContainsRemediatedProductPackage":false,"ContainsPreTreatedProductPackage":false,"IsVoided":false,"CreatedDateTime":"2026-08-27T13:59:46+00:00","CreatedByUserName":"Pablo Dayton","LastModified":"2026-08-27T13:59:46+00:00","DeliveryId":0,"RecipientFacilityLicenseNumber":null,"RecipientFacilityName":null,"ShipmentTypeName":null,"ShipmentTransactionType":null,"EstimatedDepartureDateTime":"0001-01-01T00:00:00.000","ActualDepartureDateTime":null,"EstimatedArrivalDateTime":"0001-01-01T00:00:00.000","ActualArrivalDateTime":null,"DeliveryPackageCount":0,"DeliveryReceivedPackageCount":0,"ReceivedDateTime":null,"EstimatedReturnDepartureDateTime":null,"ActualReturnDepartureDateTime":null,"EstimatedReturnArrivalDateTime":null,"ActualReturnArrivalDateTime":null,"OriginatingTemplateId":null},{"Id":15908,"ManifestNumber":"T-0000015908","InvoiceNumber":"INV-B-0827-1359","ShipmentLicenseType":"Licensed","ShipperFacilityLicenseNumber":"SF-SBX-NY-3-30301","ShipperFacilityName":"Sandbox AU Cultivator","Name":"TP Template B 0827-1359","TransporterFacilityLicenseNumber":null,"TransporterFacilityName":null,"DriverName":null,"DriverOccupationalLicenseNumber":null,"DriverVehicleLicenseNumber":null,"VehicleMake":null,"VehicleModel":null,"VehicleLicensePlateNumber":null,"VehicleRegistrationNumber":null,"DeliveryCount":1,"ReceivedDeliveryCount":0,"PackageCount":0,"ReceivedPackageCount":0,"ContainsPlantPackage":false,"ContainsProductPackage":false,"ContainsTradeSample":false,"ContainsDonation":false,"ContainsTestingSample":false,"ContainsProductRequiresRemediation":false,"ContainsRemediatedProductPackage":false,"ContainsPreTreatedProductPackage":false,"IsVoided":false,"CreatedDateTime":"2026-08-27T13:59:46+00:00","CreatedByUserName":"Pablo Dayton","LastModified":"2026-08-27T13:59:46+00:00","DeliveryId":0,"RecipientFacilityLicenseNumber":null,"RecipientFacilityName":null,"ShipmentTypeName":null,"ShipmentTransactionType":null,"EstimatedDepartureDateTime":"0001-01-01T00:00:00.000","ActualDepartureDateTime":null,"EstimatedArrivalDateTime":"0001-01-01T00:00:00.000","ActualArrivalDateTime":null,"DeliveryPackageCount":0,"DeliveryReceivedPackageCount":0,"ReceivedDateTime":null,"EstimatedReturnDepartureDateTime":null,"ActualReturnDepartureDateTime":null,"EstimatedReturnArrivalDateTime":null,"ActualReturnArrivalDateTime":null,"OriginatingTemplateId":null},{"Id":15906,"ManifestNumber":"T-0000015906","InvoiceNumber":"INV-B-0827-1358","ShipmentLicenseType":"Licensed","ShipperFacilityLicenseNumber":"SF-SBX-NY-3-30301","ShipperFacilityName":"Sandbox AU Cultivator","Name":"TP Template B 0827-1358","TransporterFacilityLicenseNumber":null,"TransporterFacilityName":null,"DriverName":null,"DriverOccupationalLicenseNumber":null,"DriverVehicleLicenseNumber":null,"VehicleMake":null,"VehicleModel":null,"VehicleLicensePlateNumber":null,"VehicleRegistrationNumber":null,"DeliveryCount":1,"ReceivedDeliveryCount":0,"PackageCount":0,"ReceivedPackageCount":0,"ContainsPlantPackage":false,"ContainsProductPackage":false,"ContainsTradeSample":false,"ContainsDonation":false,"ContainsTestingSample":false,"ContainsProductRequiresRemediation":false,"ContainsRemediatedProductPackage":false,"ContainsPreTreatedProductPackage":false,"IsVoided":false,"CreatedDateTime":"2026-08-27T13:59:06+00:00","CreatedByUserName":"Pablo Dayton","LastModified":"2026-08-27T13:59:06+00:00","DeliveryId":0,"RecipientFacilityLicenseNumber":null,"RecipientFacilityName":null,"ShipmentTypeName":null,"ShipmentTransactionType":null,"EstimatedDepartureDateTime":"0001-01-01T00:00:00.000","ActualDepartureDateTime":null,"EstimatedArrivalDateTime":"0001-01-01T00:00:00.000","ActualArrivalDateTime":null,"DeliveryPackageCount":0,"DeliveryReceivedPackageCount":0,"ReceivedDateTime":null,"EstimatedReturnDepartureDateTime":null,"ActualReturnDepartureDateTime":null,"EstimatedReturnArrivalDateTime":null,"ActualReturnArrivalDateTime":null,"OriginatingTemplateId":null},{"Id":16004,"ManifestNumber":"T-0000016004","InvoiceNumber":"INV-A-0827-1358","ShipmentLicenseType":"Licensed","ShipperFacilityLicenseNumber":"SF-SBX-NY-3-30301","ShipperFacilityName":"Sandbox AU Cultivator","Name":"TP Template A 0827-1358 (Updated)","TransporterFacilityLicenseNumber":null,"TransporterFacilityName":null,"DriverName":null,"DriverOccupationalLicenseNumber":null,"DriverVehicleLicenseNumber":null,"VehicleMake":null,"VehicleModel":null,"VehicleLicensePlateNumber":null,"VehicleRegistrationNumber":null,"DeliveryCount":1,"ReceivedDeliveryCount":0,"PackageCount":0,"ReceivedPackageCount":0,"ContainsPlantPackage":false,"ContainsProductPackage":false,"ContainsTradeSample":false,"ContainsDonation":false,"ContainsTestingSample":false,"ContainsProductRequiresRemediation":false,"ContainsRemediatedProductPackage":false,"ContainsPreTreatedProductPackage":false,"IsVoided":false,"CreatedDateTime":"2026-08-27T13:59:06+00:00","CreatedByUserName":"Pablo Dayton","LastModified":"2026-08-27T13:59:07+00:00","DeliveryId":0,"RecipientFacilityLicenseNumber":null,"RecipientFacilityName":null,"ShipmentTypeName":null,"ShipmentTransactionType":null,"EstimatedDepartureDateTime":"0001-01-01T00:00:00.000","ActualDepartureDateTime":null,"EstimatedArrivalDateTime":"0001-01-01T00:00:00.000","ActualArrivalDateTime":null,"DeliveryPackageCount":0,"DeliveryReceivedPackageCount":0,"ReceivedDateTime":null,"EstimatedReturnDepartureDateTime":null,"ActualReturnDepartureDateTime":null,"EstimatedReturnArrivalDateTime":null,"ActualReturnArrivalDateTime":null,"OriginatingTemplateId":null},{"Id":15905,"ManifestNumber":"T-0000015905","InvoiceNumber":"INV-B-0827-1357","ShipmentLicenseType":"Licensed","ShipperFacilityLicenseNumber":"SF-SBX-NY-3-30301","ShipperFacilityName":"Sandbox AU Cultivator","Name":"TP Template B 0827-1357","TransporterFacilityLicenseNumber":null,"TransporterFacilityName":null,"DriverName":null,"DriverOccupationalLicenseNumber":null,"DriverVehicleLicenseNumber":null,"VehicleMake":null,"VehicleModel":null,"VehicleLicensePlateNumber":null,"VehicleRegistrationNumber":null,"DeliveryCount":1,"ReceivedDeliveryCount":0,"PackageCount":0,"ReceivedPackageCount":0,"ContainsPlantPackage":false,"ContainsProductPackage":false,"ContainsTradeSample":false,"ContainsDonation":false,"ContainsTestingSample":false,"ContainsProductRequiresRemediation":false,"ContainsRemediatedProductPackage":false,"ContainsPreTreatedProductPackage":false,"IsVoided":false,"CreatedDateTime":"2026-08-27T13:57:53+00:00","CreatedByUserName":"Pablo Dayton","LastModified":"2026-08-27T13:57:53+00:00","DeliveryId":0,"RecipientFacilityLicenseNumber":null,"RecipientFacilityName":null,"ShipmentTypeName":null,"ShipmentTransactionType":null,"EstimatedDepartureDateTime":"0001-01-01T00:00:00.000","ActualDepartureDateTime":null,"EstimatedArrivalDateTime":"0001-01-01T00:00:00.000","ActualArrivalDateTime":null,"DeliveryPackageCount":0,"DeliveryReceivedPackageCount":0,"ReceivedDateTime":null,"EstimatedReturnDepartureDateTime":null,"ActualReturnDepartureDateTime":null,"EstimatedReturnArrivalDateTime":null,"ActualReturnArrivalDateTime":null,"OriginatingTemplateId":null},{"Id":16003,"ManifestNumber":"T-0000016003","InvoiceNumber":"INV-A-0827-1357","ShipmentLicenseType":"Licensed","ShipperFacilityLicenseNumber":"SF-SBX-NY-3-30301","ShipperFacilityName":"Sandbox AU Cultivator","Name":"TP Template A 0827-1357 (Updated)","TransporterFacilityLicenseNumber":null,"TransporterFacilityName":null,"DriverName":null,"DriverOccupationalLicenseNumber":null,"DriverVehicleLicenseNumber":null,"VehicleMake":null,"VehicleModel":null,"VehicleLicensePlateNumber":null,"VehicleRegistrationNumber":null,"DeliveryCount":1,"ReceivedDeliveryCount":0,"PackageCount":0,"ReceivedPackageCount":0,"ContainsPlantPackage":false,"ContainsProductPackage":false,"ContainsTradeSample":false,"ContainsDonation":false,"ContainsTestingSample":false,"ContainsProductRequiresRemediation":false,"ContainsRemediatedProductPackage":false,"ContainsPreTreatedProductPackage":false,"IsVoided":false,"CreatedDateTime":"2026-08-27T13:57:53+00:00","CreatedByUserName":"Pablo Dayton","LastModified":"2026-08-27T13:57:53+00:00","DeliveryId":0,"RecipientFacilityLicenseNumber":null,"RecipientFacilityName":null,"ShipmentTypeName":null,"ShipmentTransactionType":null,"EstimatedDepartureDateTime":"0001-01-01T00:00:00.000","ActualDepartureDateTime":null,"EstimatedArrivalDateTime":"0001-01-01T00:00:00.000","ActualArrivalDateTime":null,"DeliveryPackageCount":0,"DeliveryReceivedPackageCount":0,"ReceivedDateTime":null,"EstimatedReturnDepartureDateTime":null,"ActualReturnDepartureDateTime":null,"EstimatedReturnArrivalDateTime":null,"ActualReturnArrivalDateTime":null,"OriginatingTemplateId":null},{"Id":15903,"ManifestNumber":"T-0000015903","InvoiceNumber":"INV-A-0827-1355","ShipmentLicenseType":"Licensed","ShipperFacilityLicenseNumber":"SF-SBX-NY-3-30301","ShipperFacilityName":"Sandbox AU Cultivator","Name":"TP Template A 0827-1355 (Updated)","TransporterFacilityLicenseNumber":null,"TransporterFacilityName":null,"DriverName":null,"DriverOccupationalLicenseNumber":null,"DriverVehicleLicenseNumber":null,"VehicleMake":null,"VehicleModel":null,"VehicleLicensePlateNumber":null,"VehicleRegistrationNumber":null,"DeliveryCount":1,"ReceivedDeliveryCount":0,"PackageCount":0,"ReceivedPackageCount":0,"ContainsPlantPackage":false,"ContainsProductPackage":false,"ContainsTradeSample":false,"ContainsDonation":false,"ContainsTestingSample":false,"ContainsProductRequiresRemediation":false,"ContainsRemediatedProductPackage":false,"ContainsPreTreatedProductPackage":false,"IsVoided":false,"CreatedDateTime":"2026-08-27T13:56:00+00:00","CreatedByUserName":"Pablo Dayton","LastModified":"2026-08-27T13:56:01+00:00","DeliveryId":0,"RecipientFacilityLicenseNumber":null,"RecipientFacilityName":null,"ShipmentTypeName":null,"ShipmentTransactionType":null,"EstimatedDepartureDateTime":"0001-01-01T00:00:00.000","ActualDepartureDateTime":null,"EstimatedArrivalDateTime":"0001-01-01T00:00:00.000","ActualArrivalDateTime":null,"DeliveryPackageCount":0,"DeliveryReceivedPackageCount":0,"ReceivedDateTime":null,"EstimatedReturnDepartureDateTime":null,"ActualReturnDepartureDateTime":null,"EstimatedReturnArrivalDateTime":null,"ActualReturnArrivalDateTime":null,"OriginatingTemplateId":null},{"Id":15904,"ManifestNumber":"T-0000015904","InvoiceNumber":"INV-B-0827-1355","ShipmentLicenseType":"Licensed","ShipperFacilityLicenseNumber":"SF-SBX-NY-3-30301","ShipperFacilityName":"Sandbox AU Cultivator","Name":"TP Template B 0827-1355","TransporterFacilityLicenseNumber":null,"TransporterFacilityName":null,"DriverName":null,"DriverOccupationalLicenseNumber":null,"DriverVehicleLicenseNumber":null,"VehicleMake":null,"VehicleModel":null,"VehicleLicensePlateNumber":null,"VehicleRegistrationNumber":null,"DeliveryCount":1,"ReceivedDeliveryCount":0,"PackageCount":0,"ReceivedPackageCount":0,"ContainsPlantPackage":false,"ContainsProductPackage":false,"ContainsTradeSample":false,"ContainsDonation":false,"ContainsTestingSample":false,"ContainsProductRequiresRemediation":false,"ContainsRemediatedProductPackage":false,"ContainsPreTreatedProductPackage":false,"IsVoided":false,"CreatedDateTime":"2026-08-27T13:56:00+00:00","CreatedByUserName":"Pablo Dayton","LastModified":"2026-08-27T13:56:00+00:00","DeliveryId":0,"RecipientFacilityLicenseNumber":null,"RecipientFacilityName":null,"ShipmentTypeName":null,"ShipmentTransactionType":null,"EstimatedDepartureDateTime":"0001-01-01T00:00:00.000","ActualDepartureDateTime":null,"EstimatedArrivalDateTime":"0001-01-01T00:00:00.000","ActualArrivalDateTime":null,"DeliveryPackageCount":0,"DeliveryReceivedPackageCount":0,"ReceivedDateTime":null,"EstimatedReturnDepartureDateTime":null,"ActualReturnDepartureDateTime":null,"EstimatedReturnArrivalDateTime":null,"ActualReturnArrivalDateTime":null,"OriginatingTemplateId":null},{"Id":15902,"ManifestNumber":"T-0000015902","InvoiceNumber":"INV-A-0827-1353","ShipmentLicenseType":"Licensed","ShipperFacilityLicenseNumber":"SF-SBX-NY-3-30301","ShipperFacilityName":"Sandbox AU Cultivator","Name":"TP Template A 0827-1353 (Updated)","TransporterFacilityLicenseNumber":null,"TransporterFacilityName":null,"DriverName":null,"DriverOccupationalLicenseNumber":null,"DriverVehicleLicenseNumber":null,"VehicleMake":null,"VehicleModel":null,"VehicleLicensePlateNumber":null,"VehicleRegistrationNumber":null,"DeliveryCount":1,"ReceivedDeliveryCount":0,"PackageCount":0,"ReceivedPackageCount":0,"ContainsPlantPackage":false,"ContainsProductPackage":false,"ContainsTradeSample":false,"ContainsDonation":false,"ContainsTestingSample":false,"ContainsProductRequiresRemediation":false,"ContainsRemediatedProductPackage":false,"ContainsPreTreatedProductPackage":false,"IsVoided":false,"CreatedDateTime":"2026-08-27T13:54:08+00:00","CreatedByUserName":"Pablo Dayton","LastModified":"2026-08-27T13:54:08+00:00","DeliveryId":0,"RecipientFacilityLicenseNumber":null,"RecipientFacilityName":null,"ShipmentTypeName":null,"ShipmentTransactionType":null,"EstimatedDepartureDateTime":"0001-01-01T00:00:00.000","ActualDepartureDateTime":null,"EstimatedArrivalDateTime":"0001-01-01T00:00:00.000","ActualArrivalDateTime":null,"DeliveryPackageCount":0,"DeliveryReceivedPackageCount":0,"ReceivedDateTime":null,"EstimatedReturnDepartureDateTime":null,"ActualReturnDepartureDateTime":null,"EstimatedReturnArrivalDateTime":null,"ActualReturnArrivalDateTime":null,"OriginatingTemplateId":null},{"Id":16002,"ManifestNumber":"T-0000016002","InvoiceNumber":"INV-B-0827-1353","ShipmentLicenseType":"Licensed","ShipperFacilityLicenseNumber":"SF-SBX-NY-3-30301","ShipperFacilityName":"Sandbox AU Cultivator","Name":"TP Template B 0827-1353","TransporterFacilityLicenseNumber":null,"TransporterFacilityName":null,"DriverName":null,"DriverOccupationalLicenseNumber":null,"DriverVehicleLicenseNumber":null,"VehicleMake":null,"VehicleModel":null,"VehicleLicensePlateNumber":null,"VehicleRegistrationNumber":null,"DeliveryCount":1,"ReceivedDeliveryCount":0,"PackageCount":0,"ReceivedPackageCount":0,"ContainsPlantPackage":false,"ContainsProductPackage":false,"ContainsTradeSample":false,"ContainsDonation":false,"ContainsTestingSample":false,"ContainsProductRequiresRemediation":false,"ContainsRemediatedProductPackage":false,"ContainsPreTreatedProductPackage":false,"IsVoided":false,"CreatedDateTime":"2026-08-27T13:54:08+00:00","CreatedByUserName":"Pablo Dayton","LastModified":"2026-08-27T13:54:08+00:00","DeliveryId":0,"RecipientFacilityLicenseNumber":null,"RecipientFacilityName":null,"ShipmentTypeName":null,"ShipmentTransactionType":null,"EstimatedDepartureDateTime":"0001-01-01T00:00:00.000","ActualDepartureDateTime":null,"EstimatedArrivalDateTime":"0001-01-01T00:00:00.000","ActualArrivalDateTime":null,"DeliveryPackageCount":0,"DeliveryReceivedPackageCount":0,"ReceivedDateTime":null,"EstimatedReturnDepartureDateTime":null,"ActualReturnDepartureDateTime":null,"EstimatedReturnArrivalDateTime":null,"ActualReturnArrivalDateTime":null,"OriginatingTemplateId":null}],"Total":14,"TotalRecords":14,"PageSize":14,"RecordsOnPage":14,"Page":1,"CurrentPage":1,"TotalPages":1}</t>
+          <t>{"Data":[{"Id":15910,"ManifestNumber":"T-0000015910","InvoiceNumber":"INV-A-0829-1332","ShipmentLicenseType":"Licensed","ShipperFacilityLicenseNumber":"SF-SBX-NY-3-30301","ShipperFacilityName":"Sandbox AU Cultivator","Name":"TP Template A 0829-1332","TransporterFacilityLicenseNumber":null,"TransporterFacilityName":null,"DriverName":null,"DriverOccupationalLicenseNumber":null,"DriverVehicleLicenseNumber":null,"VehicleMake":null,"VehicleModel":null,"VehicleLicensePlateNumber":null,"VehicleRegistrationNumber":null,"DeliveryCount":1,"ReceivedDeliveryCount":0,"PackageCount":0,"ReceivedPackageCount":0,"ContainsPlantPackage":false,"ContainsProductPackage":false,"ContainsTradeSample":false,"ContainsDonation":false,"ContainsTestingSample":false,"ContainsProductRequiresRemediation":false,"ContainsRemediatedProductPackage":false,"ContainsPreTreatedProductPackage":false,"IsVoided":false,"CreatedDateTime":"2026-08-29T13:32:25+00:00","CreatedByUserName":"Pablo Dayton","LastModified":"2026-08-29T13:32:25+00:00","DeliveryId":0,"RecipientFacilityLicenseNumber":null,"RecipientFacilityName":null,"ShipmentTypeName":null,"ShipmentTransactionType":null,"EstimatedDepartureDateTime":"0001-01-01T00:00:00.000","ActualDepartureDateTime":null,"EstimatedArrivalDateTime":"0001-01-01T00:00:00.000","ActualArrivalDateTime":null,"DeliveryPackageCount":0,"DeliveryReceivedPackageCount":0,"ReceivedDateTime":null,"EstimatedReturnDepartureDateTime":null,"ActualReturnDepartureDateTime":null,"EstimatedReturnArrivalDateTime":null,"ActualReturnArrivalDateTime":null,"OriginatingTemplateId":null},{"Id":15911,"ManifestNumber":"T-0000015911","InvoiceNumber":"INV-B-0829-1332","ShipmentLicenseType":"Licensed","ShipperFacilityLicenseNumber":"SF-SBX-NY-3-30301","ShipperFacilityName":"Sandbox AU Cultivator","Name":"TP Template B 0829-1332","TransporterFacilityLicenseNumber":null,"TransporterFacilityName":null,"DriverName":null,"DriverOccupationalLicenseNumber":null,"DriverVehicleLicenseNumber":null,"VehicleMake":null,"VehicleModel":null,"VehicleLicensePlateNumber":null,"VehicleRegistrationNumber":null,"DeliveryCount":1,"ReceivedDeliveryCount":0,"PackageCount":0,"ReceivedPackageCount":0,"ContainsPlantPackage":false,"ContainsProductPackage":false,"ContainsTradeSample":false,"ContainsDonation":false,"ContainsTestingSample":false,"ContainsProductRequiresRemediation":false,"ContainsRemediatedProductPackage":false,"ContainsPreTreatedProductPackage":false,"IsVoided":false,"CreatedDateTime":"2026-08-29T13:32:25+00:00","CreatedByUserName":"Pablo Dayton","LastModified":"2026-08-29T13:32:25+00:00","DeliveryId":0,"RecipientFacilityLicenseNumber":null,"RecipientFacilityName":null,"ShipmentTypeName":null,"ShipmentTransactionType":null,"EstimatedDepartureDateTime":"0001-01-01T00:00:00.000","ActualDepartureDateTime":null,"EstimatedArrivalDateTime":"0001-01-01T00:00:00.000","ActualArrivalDateTime":null,"DeliveryPackageCount":0,"DeliveryReceivedPackageCount":0,"ReceivedDateTime":null,"EstimatedReturnDepartureDateTime":null,"ActualReturnDepartureDateTime":null,"EstimatedReturnArrivalDateTime":null,"ActualReturnArrivalDateTime":null,"OriginatingTemplateId":null}],"Total":2,"TotalRecords":2,"PageSize":2,"RecordsOnPage":2,"Page":1,"CurrentPage":1,"TotalPages":1}</t>
         </is>
       </c>
     </row>
@@ -11372,12 +11372,12 @@
       </c>
       <c r="D17" s="248" t="inlineStr">
         <is>
-          <t>16006</t>
+          <t>15910</t>
         </is>
       </c>
       <c r="E17" s="250" t="inlineStr">
         <is>
-          <t>2026-08-27T14:02:18Z</t>
+          <t>2026-08-29T13:32:25Z</t>
         </is>
       </c>
       <c r="F17" s="247" t="inlineStr">
@@ -11387,12 +11387,12 @@
       </c>
       <c r="G17" s="247" t="inlineStr">
         <is>
-          <t>https://sandbox-api-ny.metrc.com/transfers/v2/templates/outgoing/16006/deliveries</t>
+          <t>https://sandbox-api-ny.metrc.com/transfers/v2/templates/outgoing/15910/deliveries</t>
         </is>
       </c>
       <c r="H17" s="262" t="inlineStr">
         <is>
-          <t>{"Data":[{"Id":16511,"ManifestNumber":null,"DeliveryNumber":0,"RecipientFacilityLicenseNumber":"SF-SBX-NY-5-30301","RecipientFacilityName":"Sandbox AU Dispensary","ShipmentTypeName":"Affiliated Transfer","ShipmentTransactionType":"Standard","InvoiceNumber":"INV-A-0827-1402","PaymentTermDays":null,"PaymentDueDate":null,"EstimatedDepartureDateTime":"2026-08-27T15:02:00.000","ActualDepartureDateTime":null,"EstimatedArrivalDateTime":"2026-08-27T18:02:00.000","ActualArrivalDateTime":null,"GrossWeight":null,"GrossUnitOfWeightId":null,"GrossUnitOfWeightName":null,"PlannedRoute":"Evaluation route.","DeliveryPackageCount":0,"DeliveryReceivedPackageCount":0,"ReceivedDateTime":null,"EstimatedReturnDepartureDateTime":null,"ActualReturnDepartureDateTime":null,"EstimatedReturnArrivalDateTime":null,"ActualReturnArrivalDateTime":null,"RejectedPackagesReturned":false,"PDFDocumentFileSystemId":null}],"Total":1,"TotalRecords":1,"PageSize":1,"RecordsOnPage":1,"Page":1,"CurrentPage":1,"TotalPages":1}</t>
+          <t>{"Data":[{"Id":16412,"ManifestNumber":null,"DeliveryNumber":0,"RecipientFacilityLicenseNumber":"SF-SBX-NY-6-13402","RecipientFacilityName":"Sandbox AU Distributor","ShipmentTypeName":"Unaffiliated Transfer","ShipmentTransactionType":"Wholesale","InvoiceNumber":"INV-A-0829-1332","PaymentTermDays":null,"PaymentDueDate":null,"EstimatedDepartureDateTime":"2026-08-29T14:32:00.000","ActualDepartureDateTime":null,"EstimatedArrivalDateTime":"2026-08-29T17:32:00.000","ActualArrivalDateTime":null,"GrossWeight":null,"GrossUnitOfWeightId":null,"GrossUnitOfWeightName":null,"PlannedRoute":"Evaluation route.","DeliveryPackageCount":0,"DeliveryReceivedPackageCount":0,"ReceivedDateTime":null,"EstimatedReturnDepartureDateTime":null,"ActualReturnDepartureDateTime":null,"EstimatedReturnArrivalDateTime":null,"ActualReturnArrivalDateTime":null,"RejectedPackagesReturned":false,"PDFDocumentFileSystemId":null}],"Total":1,"TotalRecords":1,"PageSize":1,"RecordsOnPage":1,"Page":1,"CurrentPage":1,"TotalPages":1}</t>
         </is>
       </c>
     </row>
@@ -11452,12 +11452,12 @@
       </c>
       <c r="D21" s="248" t="inlineStr">
         <is>
-          <t>16006</t>
+          <t>15910</t>
         </is>
       </c>
       <c r="E21" s="250" t="inlineStr">
         <is>
-          <t>2026-08-27T14:02:18Z</t>
+          <t>2026-08-29T13:32:26Z</t>
         </is>
       </c>
       <c r="F21" s="247" t="inlineStr">
@@ -11472,7 +11472,7 @@
       </c>
       <c r="H21" s="262" t="inlineStr">
         <is>
-          <t>[{"Name":"TP Template A 0827-1402 (Updated)","TransporterFacilityLicenseNumber":null,"DriverOccupationalLicenseNumber":null,"DriverName":null,"DriverLicenseNumber":null,"PhoneNumberForQuestions":null,"VehicleMake":null,"VehicleModel":null,"VehicleLicensePlateNumber":null,"VehicleRegistrationNumber":null,"Destinations":[{"RecipientLicenseNumber":"SF-SBX-NY-5-30301","InvoiceNumber":"INV-A-0827-1402","TransferTypeName":"Affiliated Transfer","PlannedRoute":"Evaluation route.","EstimatedDepartureDateTime":"2026-08-27T15:02:16Z","EstimatedArrivalDateTime":"2026-08-27T18:02:16Z","Transporters":[],"Packages":[],"TransferDestinationId":0}],"TransferTemplateId":16006}]</t>
+          <t>[{"Name":"TP Template A 0829-1332 (Updated)","TransporterFacilityLicenseNumber":null,"DriverOccupationalLicenseNumber":null,"DriverName":null,"DriverLicenseNumber":null,"PhoneNumberForQuestions":null,"VehicleMake":null,"VehicleModel":null,"VehicleLicensePlateNumber":null,"VehicleRegistrationNumber":null,"Destinations":[{"RecipientLicenseNumber":"SF-SBX-NY-6-13402","InvoiceNumber":"INV-A-0829-1332","TransferTypeName":"Unaffiliated Transfer","PlannedRoute":"Evaluation route.","EstimatedDepartureDateTime":"2026-08-29T14:32:24Z","EstimatedArrivalDateTime":"2026-08-29T17:32:24Z","Transporters":[],"Packages":[],"TransferDestinationId":0}],"TransferTemplateId":15910}]</t>
         </is>
       </c>
     </row>
@@ -11853,7 +11853,7 @@
       </c>
       <c r="E5" s="250" t="inlineStr">
         <is>
-          <t>2026-08-27T14:02:18Z</t>
+          <t>2026-08-29T13:32:26Z</t>
         </is>
       </c>
       <c r="F5" s="247" t="inlineStr">
@@ -11868,7 +11868,7 @@
       </c>
       <c r="H5" s="262" t="inlineStr">
         <is>
-          <t>[{"ShipperLicenseNumber":"SF-SBX-NY-5-30301","ShipperName":"Evaluation Shipper","ShipperMainPhoneNumber":"555-000-0000","ShipperAddress1":"1 Evaluation Way","ShipperAddress2":null,"ShipperAddressCity":"Albany","ShipperAddressState":"NY","ShipperAddressPostalCode":"12207","TransporterFacilityLicenseNumber":null,"DriverOccupationalLicenseNumber":null,"DriverName":null,"DriverLicenseNumber":null,"PhoneNumberForQuestions":null,"VehicleMake":null,"VehicleModel":null,"VehicleLicensePlateNumber":null,"VehicleRegistrationNumber":null,"Destinations":[{"RecipientLicenseNumber":"SF-SBX-NY-3-30301","InvoiceNumber":"EXT-A-0827-1402","TransferTypeName":"Beginning Inventory","PlannedRoute":"Evaluation route.","EstimatedDepartureDateTime":"2026-08-27T15:02:18Z","EstimatedArrivalDateTime":"2026-08-27T18:02:18Z","GrossWeight":null,"GrossUnitOfWeightId":null,"Transporters":[],"Packages":[]}]}]</t>
+          <t>[{"ShipperLicenseNumber":"SF-SBX-NY-6-13402","ShipperName":"Evaluation Shipper","ShipperMainPhoneNumber":"555-000-0000","ShipperAddress1":"1 Evaluation Way","ShipperAddress2":null,"ShipperAddressCity":"Albany","ShipperAddressState":"NY","ShipperAddressPostalCode":"12207","TransporterFacilityLicenseNumber":null,"DriverOccupationalLicenseNumber":null,"DriverName":null,"DriverLicenseNumber":null,"PhoneNumberForQuestions":null,"VehicleMake":null,"VehicleModel":null,"VehicleLicensePlateNumber":null,"VehicleRegistrationNumber":null,"Destinations":[{"RecipientLicenseNumber":"SF-SBX-NY-3-30301","InvoiceNumber":"EXT-A-0829-1332","TransferTypeName":"Beginning Inventory","PlannedRoute":"Evaluation route.","EstimatedDepartureDateTime":"2026-08-29T14:32:26Z","EstimatedArrivalDateTime":"2026-08-29T17:32:26Z","GrossWeight":null,"GrossUnitOfWeightId":null,"Transporters":[],"Packages":[]}]}]</t>
         </is>
       </c>
     </row>
@@ -11927,7 +11927,7 @@
       </c>
       <c r="E9" s="250" t="inlineStr">
         <is>
-          <t>2026-08-27T14:02:18Z</t>
+          <t>2026-08-29T13:32:26Z</t>
         </is>
       </c>
       <c r="F9" s="247" t="inlineStr">
@@ -11942,7 +11942,7 @@
       </c>
       <c r="H9" s="262" t="inlineStr">
         <is>
-          <t>[{"ShipperLicenseNumber":"SF-SBX-NY-5-30301","ShipperName":"Evaluation Shipper","ShipperMainPhoneNumber":"555-000-0000","ShipperAddress1":"1 Evaluation Way","ShipperAddress2":null,"ShipperAddressCity":"Albany","ShipperAddressState":"NY","ShipperAddressPostalCode":"12207","TransporterFacilityLicenseNumber":null,"DriverOccupationalLicenseNumber":null,"DriverName":null,"DriverLicenseNumber":null,"PhoneNumberForQuestions":null,"VehicleMake":null,"VehicleModel":null,"VehicleLicensePlateNumber":null,"VehicleRegistrationNumber":null,"Destinations":[{"RecipientLicenseNumber":"SF-SBX-NY-3-30301","InvoiceNumber":"EXT-B-0827-1402","TransferTypeName":"Beginning Inventory","PlannedRoute":"Evaluation route.","EstimatedDepartureDateTime":"2026-08-27T15:02:18Z","EstimatedArrivalDateTime":"2026-08-27T18:02:18Z","GrossWeight":null,"GrossUnitOfWeightId":null,"Transporters":[],"Packages":[]}]}]</t>
+          <t>[{"ShipperLicenseNumber":"SF-SBX-NY-6-13402","ShipperName":"Evaluation Shipper","ShipperMainPhoneNumber":"555-000-0000","ShipperAddress1":"1 Evaluation Way","ShipperAddress2":null,"ShipperAddressCity":"Albany","ShipperAddressState":"NY","ShipperAddressPostalCode":"12207","TransporterFacilityLicenseNumber":null,"DriverOccupationalLicenseNumber":null,"DriverName":null,"DriverLicenseNumber":null,"PhoneNumberForQuestions":null,"VehicleMake":null,"VehicleModel":null,"VehicleLicensePlateNumber":null,"VehicleRegistrationNumber":null,"Destinations":[{"RecipientLicenseNumber":"SF-SBX-NY-3-30301","InvoiceNumber":"EXT-B-0829-1332","TransferTypeName":"Beginning Inventory","PlannedRoute":"Evaluation route.","EstimatedDepartureDateTime":"2026-08-29T14:32:26Z","EstimatedArrivalDateTime":"2026-08-29T17:32:26Z","GrossWeight":null,"GrossUnitOfWeightId":null,"Transporters":[],"Packages":[]}]}]</t>
         </is>
       </c>
     </row>
@@ -12000,7 +12000,7 @@
       </c>
       <c r="E13" s="250" t="inlineStr">
         <is>
-          <t>2026-08-27T14:02:18Z</t>
+          <t>2026-08-29T13:32:26Z</t>
         </is>
       </c>
       <c r="F13" s="247" t="inlineStr">
@@ -12010,7 +12010,7 @@
       </c>
       <c r="G13" s="247" t="inlineStr">
         <is>
-          <t>https://sandbox-api-ny.metrc.com/transfers/v2/incoming?lastModifiedStart=2026-08-26T14%3A02%3A18Z&amp;lastModifiedEnd=2026-08-27T14%3A02%3A18Z&amp;licenseNumber=SF-SBX-NY-3-30301</t>
+          <t>https://sandbox-api-ny.metrc.com/transfers/v2/incoming?lastModifiedStart=2026-08-28T13%3A32%3A26Z&amp;lastModifiedEnd=2026-08-29T13%3A32%3A26Z&amp;licenseNumber=SF-SBX-NY-3-30301</t>
         </is>
       </c>
       <c r="H13" s="262" t="inlineStr">

</xml_diff>

<commit_message>
Stop depending on data the sandbox happens to already hold
The sandbox was reset between runs, which exposed two places where tabs relied
on pre-existing data rather than creating what they need.

The Plants tab needs flowering plants, but nothing produces any: the
PlantBatches tab moves its plants to Vegetative because that is what its step 3
asks for, then destroys the remainder. It only ever passed because the sandbox
already contained flowering plants. It now grows a batch and phases it to
Flowering as setup.

Seeding a dispensary picked an item category requiring a strain and passed none
when the facility had no strains, which a reset guarantees. It now creates one
first.

Both failures were invisible until the reset, and neither would have reproduced
on a fresh evaluator's sandbox.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WckmkszE5f38nyn3gphdpj
</commit_message>
<xml_diff>
--- a/evidence/metrc/Evaluation_NY_completed.xlsx
+++ b/evidence/metrc/Evaluation_NY_completed.xlsx
@@ -2449,12 +2449,12 @@
       </c>
       <c r="D5" s="248" t="inlineStr">
         <is>
-          <t>59123</t>
+          <t>59017</t>
         </is>
       </c>
       <c r="E5" s="250" t="inlineStr">
         <is>
-          <t>2026-08-27T14:02:09Z</t>
+          <t>2026-08-29T14:27:48Z</t>
         </is>
       </c>
       <c r="F5" s="247" t="inlineStr">
@@ -2469,7 +2469,7 @@
       </c>
       <c r="H5" s="261" t="inlineStr">
         <is>
-          <t>[{"Name":"TP Batch 0827-1402","Type":"Clone","Count":6,"Strain":"Terpenomics Strain 0827-1402","Location":"Terpenomics Loc 0827-1402 (Updated)","Sublocation":null,"PatientLicenseNumber":null,"ActualDate":"2026-08-27","SourcePlantBatches":null}]</t>
+          <t>[{"Name":"TP Batch 0829-1427","Type":"Clone","Count":6,"Strain":"Terpenomics Strain 0829-1427","Location":"Terpenomics Loc 0829-1427 (Updated)","Sublocation":null,"PatientLicenseNumber":null,"ActualDate":"2026-08-29","SourcePlantBatches":null}]</t>
         </is>
       </c>
     </row>
@@ -2529,17 +2529,17 @@
       </c>
       <c r="D9" s="248" t="inlineStr">
         <is>
-          <t>217773</t>
+          <t>218945</t>
         </is>
       </c>
       <c r="E9" s="250" t="inlineStr">
         <is>
-          <t>2026-08-27T14:02:09Z</t>
+          <t>2026-08-29T14:27:48Z</t>
         </is>
       </c>
       <c r="F9" s="247" t="inlineStr">
         <is>
-          <t>1A4120300004532000001445</t>
+          <t>1A4120300004532000001525</t>
         </is>
       </c>
       <c r="G9" s="104" t="inlineStr">
@@ -2549,7 +2549,7 @@
       </c>
       <c r="H9" s="261" t="inlineStr">
         <is>
-          <t>[{"Id":null,"PlantBatch":"TP Batch 0827-1402","Count":3,"Location":"Terpenomics Loc 0827-1402 (Updated)","Sublocation":null,"Item":"Terpenomics Clone 0827-1402","Tag":"1A4120300004532000001445","PatientLicenseNumber":null,"Note":"Evaluation step","IsTradeSample":false,"IsDonation":false,"ActualDate":"2026-08-27"}]</t>
+          <t>[{"Id":null,"PlantBatch":"TP Batch 0829-1427","Count":3,"Location":"Terpenomics Loc 0829-1427 (Updated)","Sublocation":null,"Item":"Terpenomics Clone 0829-1427","Tag":"1A4120300004532000001525","PatientLicenseNumber":null,"Note":"Evaluation step","IsTradeSample":false,"IsDonation":false,"ActualDate":"2026-08-29"}]</t>
         </is>
       </c>
     </row>
@@ -2602,17 +2602,17 @@
       </c>
       <c r="D13" s="248" t="inlineStr">
         <is>
-          <t>751530, 751531</t>
+          <t>751545, 751546</t>
         </is>
       </c>
       <c r="E13" s="250" t="inlineStr">
         <is>
-          <t>2026-08-27T14:02:09Z</t>
+          <t>2026-08-29T14:27:49Z</t>
         </is>
       </c>
       <c r="F13" s="247" t="inlineStr">
         <is>
-          <t>1A4120200004532000001595, 1A4120200004532000001596</t>
+          <t>1A4120200004532000001675, 1A4120200004532000001676</t>
         </is>
       </c>
       <c r="G13" s="104" t="inlineStr">
@@ -2622,7 +2622,7 @@
       </c>
       <c r="H13" s="261" t="inlineStr">
         <is>
-          <t>[{"Name":"TP Batch 0827-1402","Count":2,"StartingTag":"1A4120200004532000001595","GrowthPhase":"Vegetative","NewLocation":"Terpenomics Loc 0827-1402 (Updated)","NewSublocation":null,"GrowthDate":"2026-08-27","PatientLicenseNumber":null}]</t>
+          <t>[{"Name":"TP Batch 0829-1427","Count":2,"StartingTag":"1A4120200004532000001675","GrowthPhase":"Vegetative","NewLocation":"Terpenomics Loc 0829-1427 (Updated)","NewSublocation":null,"GrowthDate":"2026-08-29","PatientLicenseNumber":null}]</t>
         </is>
       </c>
     </row>
@@ -2682,12 +2682,12 @@
       </c>
       <c r="D17" s="248" t="inlineStr">
         <is>
-          <t>59123</t>
+          <t>59017</t>
         </is>
       </c>
       <c r="E17" s="250" t="inlineStr">
         <is>
-          <t>2026-08-27T14:02:09Z</t>
+          <t>2026-08-29T14:27:49Z</t>
         </is>
       </c>
       <c r="F17" s="247" t="inlineStr">
@@ -2702,7 +2702,7 @@
       </c>
       <c r="H17" s="261" t="inlineStr">
         <is>
-          <t>[{"PlantBatch":"TP Batch 0827-1402","Count":1,"WasteMethodName":null,"WasteMaterialMixed":null,"WasteReasonName":"Waste","ReasonNote":"Evaluation step — destroying one immature plant.","WasteWeight":1.0,"WasteUnitOfMeasure":"Grams","ActualDate":"2026-08-27"}]</t>
+          <t>[{"PlantBatch":"TP Batch 0829-1427","Count":1,"WasteMethodName":null,"WasteMaterialMixed":null,"WasteReasonName":"Waste","ReasonNote":"Evaluation step — destroying one immature plant.","WasteWeight":1.0,"WasteUnitOfMeasure":"Grams","ActualDate":"2026-08-29"}]</t>
         </is>
       </c>
     </row>
@@ -3075,12 +3075,12 @@
       </c>
       <c r="E6" s="250" t="inlineStr">
         <is>
-          <t>2026-08-27T14:00:21+00:00</t>
+          <t>2026-08-29T14:27:50+00:00</t>
         </is>
       </c>
       <c r="F6" s="247" t="inlineStr">
         <is>
-          <t>1A4120200004532000001006</t>
+          <t>1A4120200004532000001677</t>
         </is>
       </c>
       <c r="G6" s="104" t="n"/>
@@ -3091,7 +3091,7 @@
       </c>
       <c r="I6" s="262" t="inlineStr">
         <is>
-          <t>[{"Id":null,"Label":"1A4120200004532000001006","Location":"Terpenomics Loc 0827-1402 (Updated)","Sublocation":null,"ActualDate":"2026-08-27"}]</t>
+          <t>[{"Id":null,"Label":"1A4120200004532000001677","Location":"Terpenomics Loc 0829-1427 (Updated)","Sublocation":null,"ActualDate":"2026-08-29"}]</t>
         </is>
       </c>
     </row>
@@ -3146,22 +3146,22 @@
       </c>
       <c r="D10" s="248" t="inlineStr">
         <is>
-          <t>59124</t>
+          <t>59019</t>
         </is>
       </c>
       <c r="E10" s="250" t="inlineStr">
         <is>
-          <t>2026-08-27T14:02:10Z</t>
+          <t>2026-08-29T14:27:56Z</t>
         </is>
       </c>
       <c r="F10" s="247" t="inlineStr">
         <is>
-          <t>1A4120200004532000001006</t>
+          <t>1A4120200004532000001677</t>
         </is>
       </c>
       <c r="G10" s="104" t="inlineStr">
         <is>
-          <t>TP Immature 0827-1402</t>
+          <t>TP Immature 0829-1427</t>
         </is>
       </c>
       <c r="H10" s="247" t="inlineStr">
@@ -3171,7 +3171,7 @@
       </c>
       <c r="I10" s="262" t="inlineStr">
         <is>
-          <t>[{"PlantLabel":"1A4120200004532000001006","PlantBatchName":"TP Immature 0827-1402","PlantBatchType":"Clone","PlantCount":3,"LocationName":"Terpenomics Loc 0827-1402 (Updated)","SublocationName":null,"StrainName":"Terpenomics Strain 0827-1402","PatientLicenseNumber":null,"ActualDate":"2026-08-27T14:02:10Z"}]</t>
+          <t>[{"PlantLabel":"1A4120200004532000001677","PlantBatchName":"TP Immature 0829-1427","PlantBatchType":"Clone","PlantCount":3,"LocationName":"Terpenomics Loc 0829-1427 (Updated)","SublocationName":null,"StrainName":"Terpenomics Strain 0829-1427","PatientLicenseNumber":null,"ActualDate":"2026-08-29T14:27:56Z"}]</t>
         </is>
       </c>
     </row>
@@ -3234,17 +3234,17 @@
       </c>
       <c r="D14" s="248" t="inlineStr">
         <is>
-          <t>218906</t>
+          <t>218946</t>
         </is>
       </c>
       <c r="E14" s="250" t="inlineStr">
         <is>
-          <t>2026-08-27T14:02:10Z</t>
+          <t>2026-08-29T14:27:57Z</t>
         </is>
       </c>
       <c r="F14" s="247" t="inlineStr">
         <is>
-          <t>1A4120300004532000001446</t>
+          <t>1A4120300004532000001526</t>
         </is>
       </c>
       <c r="G14" s="104" t="n"/>
@@ -3255,7 +3255,7 @@
       </c>
       <c r="I14" s="262" t="inlineStr">
         <is>
-          <t>[{"PlantLabel":"1A4120200004532000001006","PackageTag":"1A4120300004532000001446","PlantBatchType":"Clone","Item":"Terpenomics Clone 0827-1402","Location":"Terpenomics Loc 0827-1402 (Updated)","Sublocation":null,"Note":null,"IsTradeSample":false,"PatientLicenseNumber":null,"IsDonation":false,"Count":3,"ActualDate":"2026-08-27T14:02:10Z"}]</t>
+          <t>[{"PlantLabel":"1A4120200004532000001677","PackageTag":"1A4120300004532000001526","PlantBatchType":"Clone","Item":"Terpenomics Clone 0829-1427","Location":"Terpenomics Loc 0829-1427 (Updated)","Sublocation":null,"Note":null,"IsTradeSample":false,"PatientLicenseNumber":null,"IsDonation":false,"Count":3,"ActualDate":"2026-08-29T14:27:56Z"}]</t>
         </is>
       </c>
     </row>
@@ -3318,17 +3318,17 @@
       </c>
       <c r="D18" s="248" t="inlineStr">
         <is>
-          <t>752259</t>
+          <t>750774</t>
         </is>
       </c>
       <c r="E18" s="250" t="inlineStr">
         <is>
-          <t>2026-08-27T14:02:11Z</t>
+          <t>2026-08-29T14:27:57Z</t>
         </is>
       </c>
       <c r="F18" s="247" t="inlineStr">
         <is>
-          <t>1A4120200004532000001085</t>
+          <t>1A4120200004532000001678</t>
         </is>
       </c>
       <c r="G18" s="247" t="n"/>
@@ -3339,7 +3339,7 @@
       </c>
       <c r="I18" s="262" t="inlineStr">
         <is>
-          <t>[{"Id":null,"Label":"1A4120200004532000001085","WasteMethodName":null,"WasteMaterialMixed":null,"WasteWeight":15.0,"WasteUnitOfMeasureName":"Grams","WasteReasonName":"Waste","Count":0,"ReasonNote":"Evaluation step — plant destruction.","ActualDate":"2026-08-27"}]</t>
+          <t>[{"Id":null,"Label":"1A4120200004532000001678","WasteMethodName":null,"WasteMaterialMixed":null,"WasteWeight":15.0,"WasteUnitOfMeasureName":"Grams","WasteReasonName":"Waste","Count":0,"ReasonNote":"Evaluation step — plant destruction.","ActualDate":"2026-08-29"}]</t>
         </is>
       </c>
     </row>
@@ -3401,17 +3401,17 @@
       </c>
       <c r="D22" s="248" t="inlineStr">
         <is>
-          <t>28811</t>
+          <t>28812</t>
         </is>
       </c>
       <c r="E22" s="250" t="inlineStr">
         <is>
-          <t>2026-08-27T14:02:11Z</t>
+          <t>2026-08-29T14:27:57Z</t>
         </is>
       </c>
       <c r="F22" s="247" t="inlineStr">
         <is>
-          <t>1A4120200004532000001112</t>
+          <t>1A4120200004532000001679</t>
         </is>
       </c>
       <c r="G22" s="247" t="n"/>
@@ -3422,7 +3422,7 @@
       </c>
       <c r="I22" s="262" t="inlineStr">
         <is>
-          <t>[{"Plant":"1A4120200004532000001112","Weight":25.0,"UnitOfWeight":"Grams","DryingLocation":"Terpenomics Loc 0827-1402 (Updated)","DryingSublocation":null,"HarvestName":null,"PatientLicenseNumber":null,"ActualDate":"2026-08-27","PlantCount":1}]</t>
+          <t>[{"Plant":"1A4120200004532000001679","Weight":25.0,"UnitOfWeight":"Grams","DryingLocation":"Terpenomics Loc 0829-1427 (Updated)","DryingSublocation":null,"HarvestName":null,"PatientLicenseNumber":null,"ActualDate":"2026-08-29","PlantCount":1}]</t>
         </is>
       </c>
     </row>
@@ -3484,22 +3484,22 @@
       </c>
       <c r="D26" s="248" t="inlineStr">
         <is>
-          <t>28708, 28708</t>
+          <t>28709, 28709</t>
         </is>
       </c>
       <c r="E26" s="250" t="inlineStr">
         <is>
-          <t>2026-08-27T14:02:11Z</t>
+          <t>2026-08-29T14:27:57Z</t>
         </is>
       </c>
       <c r="F26" s="247" t="inlineStr">
         <is>
-          <t>1A4120200004532000001112, 1A4120200004532000001113</t>
+          <t>1A4120200004532000001679, 1A4120200004532000001680</t>
         </is>
       </c>
       <c r="G26" s="247" t="inlineStr">
         <is>
-          <t>TP Harvest 0827-1402</t>
+          <t>TP Harvest 0829-1427</t>
         </is>
       </c>
       <c r="H26" s="247" t="inlineStr">
@@ -3509,7 +3509,7 @@
       </c>
       <c r="I26" s="262" t="inlineStr">
         <is>
-          <t>[{"Plant":"1A4120200004532000001112","Weight":100.0,"UnitOfWeight":"Grams","DryingLocation":"Terpenomics Loc 0827-1402 (Updated)","DryingSublocation":null,"HarvestName":"TP Harvest 0827-1402","PatientLicenseNumber":null,"ActualDate":"2026-08-27"},{"Plant":"1A4120200004532000001113","Weight":100.0,"UnitOfWeight":"Grams","DryingLocation":"Terpenomics Loc 0827-1402 (Updated)","DryingSublocation":null,"HarvestName":"TP Harvest 0827-1402","PatientLicenseNumber":null,"ActualDate":"2026-08-27"}]</t>
+          <t>[{"Plant":"1A4120200004532000001679","Weight":100.0,"UnitOfWeight":"Grams","DryingLocation":"Terpenomics Loc 0829-1427 (Updated)","DryingSublocation":null,"HarvestName":"TP Harvest 0829-1427","PatientLicenseNumber":null,"ActualDate":"2026-08-29"},{"Plant":"1A4120200004532000001680","Weight":100.0,"UnitOfWeight":"Grams","DryingLocation":"Terpenomics Loc 0829-1427 (Updated)","DryingSublocation":null,"HarvestName":"TP Harvest 0829-1427","PatientLicenseNumber":null,"ActualDate":"2026-08-29"}]</t>
         </is>
       </c>
     </row>
@@ -3951,22 +3951,22 @@
       </c>
       <c r="D5" s="248" t="inlineStr">
         <is>
-          <t>218907</t>
+          <t>218947</t>
         </is>
       </c>
       <c r="E5" s="250" t="inlineStr">
         <is>
-          <t>2026-08-27T14:02:11Z</t>
+          <t>2026-08-29T14:27:58Z</t>
         </is>
       </c>
       <c r="F5" s="247" t="inlineStr">
         <is>
-          <t>1A4120300004532000001447</t>
+          <t>1A4120300004532000001527</t>
         </is>
       </c>
       <c r="G5" s="104" t="inlineStr">
         <is>
-          <t>TP Harvest 0827-1402</t>
+          <t>TP Harvest 0829-1427</t>
         </is>
       </c>
       <c r="H5" s="247" t="inlineStr">
@@ -3976,7 +3976,7 @@
       </c>
       <c r="I5" s="262" t="inlineStr">
         <is>
-          <t>[{"Tag":"1A4120300004532000001447","Location":"Terpenomics Loc 0827-1402 (Updated)","Sublocation":null,"Item":"Terpenomics Item 0827-1402","UnitOfWeight":"Grams","PatientLicenseNumber":null,"Note":"Evaluation step","IsProductionBatch":false,"ProductionBatchNumber":null,"IsTradeSample":false,"IsDonation":false,"ProductRequiresRemediation":false,"RemediateProduct":false,"ActualDate":"2026-08-27","Ingredients":[{"HarvestId":28811,"HarvestName":null,"Weight":50.0,"UnitOfWeight":"Grams"}]}]</t>
+          <t>[{"Tag":"1A4120300004532000001527","Location":"Terpenomics Loc 0829-1427 (Updated)","Sublocation":null,"Item":"Terpenomics Item 0829-1427","UnitOfWeight":"Grams","PatientLicenseNumber":null,"Note":"Evaluation step","IsProductionBatch":false,"ProductionBatchNumber":null,"IsTradeSample":false,"IsDonation":false,"ProductRequiresRemediation":false,"RemediateProduct":false,"ActualDate":"2026-08-29","Ingredients":[{"HarvestId":28709,"HarvestName":null,"Weight":50.0,"UnitOfWeight":"Grams"}]}]</t>
         </is>
       </c>
     </row>
@@ -4039,12 +4039,12 @@
       </c>
       <c r="D9" s="248" t="inlineStr">
         <is>
-          <t>28811</t>
+          <t>28709</t>
         </is>
       </c>
       <c r="E9" s="250" t="inlineStr">
         <is>
-          <t>2026-08-27T14:02:12Z</t>
+          <t>2026-08-29T14:27:58Z</t>
         </is>
       </c>
       <c r="F9" s="247" t="inlineStr">
@@ -4054,7 +4054,7 @@
       </c>
       <c r="G9" s="104" t="inlineStr">
         <is>
-          <t>TP Harvest 0827-1402</t>
+          <t>TP Harvest 0829-1427</t>
         </is>
       </c>
       <c r="H9" s="247" t="inlineStr">
@@ -4064,7 +4064,7 @@
       </c>
       <c r="I9" s="262" t="inlineStr">
         <is>
-          <t>[{"Id":28811,"WasteType":"Plant Material","UnitOfWeight":"Grams","WasteWeight":25.0,"ActualDate":"2026-08-27"}]</t>
+          <t>[{"Id":28709,"WasteType":"Plant Material","UnitOfWeight":"Grams","WasteWeight":200.0,"ActualDate":"2026-08-29"}]</t>
         </is>
       </c>
     </row>
@@ -4119,12 +4119,12 @@
       </c>
       <c r="D13" s="248" t="inlineStr">
         <is>
-          <t>28811</t>
+          <t>28709</t>
         </is>
       </c>
       <c r="E13" s="250" t="inlineStr">
         <is>
-          <t>2026-08-27T14:02:12Z</t>
+          <t>2026-08-29T14:27:58Z</t>
         </is>
       </c>
       <c r="F13" s="247" t="inlineStr">
@@ -4134,7 +4134,7 @@
       </c>
       <c r="G13" s="104" t="inlineStr">
         <is>
-          <t>TP Harvest 0827-1402</t>
+          <t>TP Harvest 0829-1427</t>
         </is>
       </c>
       <c r="H13" s="247" t="inlineStr">
@@ -4144,7 +4144,7 @@
       </c>
       <c r="I13" s="262" t="inlineStr">
         <is>
-          <t>[{"Id":28811,"ActualDate":"2026-08-27"}]</t>
+          <t>[{"Id":28709,"ActualDate":"2026-08-29"}]</t>
         </is>
       </c>
     </row>
@@ -4207,12 +4207,12 @@
       </c>
       <c r="D17" s="248" t="inlineStr">
         <is>
-          <t>28811</t>
+          <t>28709</t>
         </is>
       </c>
       <c r="E17" s="250" t="inlineStr">
         <is>
-          <t>2026-08-27T14:02:12Z</t>
+          <t>2026-08-29T14:27:58Z</t>
         </is>
       </c>
       <c r="F17" s="247" t="inlineStr">
@@ -4222,7 +4222,7 @@
       </c>
       <c r="G17" s="104" t="inlineStr">
         <is>
-          <t>TP Harvest 0827-1402</t>
+          <t>TP Harvest 0829-1427</t>
         </is>
       </c>
       <c r="H17" s="247" t="inlineStr">
@@ -4232,7 +4232,7 @@
       </c>
       <c r="I17" s="262" t="inlineStr">
         <is>
-          <t>[{"Id":28811}]</t>
+          <t>[{"Id":28709}]</t>
         </is>
       </c>
     </row>
@@ -4599,17 +4599,17 @@
       </c>
       <c r="D5" s="248" t="inlineStr">
         <is>
-          <t>217774</t>
+          <t>217781</t>
         </is>
       </c>
       <c r="E5" s="250" t="inlineStr">
         <is>
-          <t>2026-08-27T14:02:12Z</t>
+          <t>2026-08-29T14:27:59Z</t>
         </is>
       </c>
       <c r="F5" s="247" t="inlineStr">
         <is>
-          <t>1A4120300004532000001448</t>
+          <t>1A4120300004532000001528</t>
         </is>
       </c>
       <c r="G5" s="247" t="inlineStr">
@@ -4619,7 +4619,7 @@
       </c>
       <c r="H5" s="262" t="inlineStr">
         <is>
-          <t>[{"Tag":"1A4120300004532000001448","Location":"Terpenomics Loc 0827-1402 (Updated)","Sublocation":null,"Item":"Terpenomics Item 0827-1402","Quantity":10.0,"UnitOfMeasure":"Grams","PatientLicenseNumber":null,"Note":"Evaluation step","IsProductionBatch":false,"ProductionBatchNumber":null,"IsDonation":false,"IsTradeSample":false,"ProductRequiresRemediation":false,"UseSameItem":true,"ActualDate":"2026-08-27","Ingredients":[{"Package":"1A4120300004532000001447","Quantity":10.0,"UnitOfMeasure":"Grams"}]}]</t>
+          <t>[{"Tag":"1A4120300004532000001528","Location":"Terpenomics Loc 0829-1427 (Updated)","Sublocation":null,"Item":"Terpenomics Item 0829-1427","Quantity":10.0,"UnitOfMeasure":"Grams","PatientLicenseNumber":null,"Note":"Evaluation step","IsProductionBatch":false,"ProductionBatchNumber":null,"IsDonation":false,"IsTradeSample":false,"ProductRequiresRemediation":false,"UseSameItem":true,"ActualDate":"2026-08-29","Ingredients":[{"Package":"1A4120300004532000001527","Quantity":10.0,"UnitOfMeasure":"Grams"}]}]</t>
         </is>
       </c>
     </row>
@@ -4684,12 +4684,12 @@
       </c>
       <c r="E9" s="250" t="inlineStr">
         <is>
-          <t>2026-08-27T14:02:12Z</t>
+          <t>2026-08-29T14:28:00Z</t>
         </is>
       </c>
       <c r="F9" s="247" t="inlineStr">
         <is>
-          <t>1A4120300004532000001448</t>
+          <t>1A4120300004532000001528</t>
         </is>
       </c>
       <c r="G9" s="247" t="inlineStr">
@@ -4699,7 +4699,7 @@
       </c>
       <c r="H9" s="262" t="inlineStr">
         <is>
-          <t>[{"Label":"1A4120300004532000001448","Item":"Terpenomics Alt Item 0827-1402"}]</t>
+          <t>[{"Label":"1A4120300004532000001528","Item":"Terpenomics Alt Item 0829-1427"}]</t>
         </is>
       </c>
     </row>
@@ -4757,12 +4757,12 @@
       </c>
       <c r="E13" s="250" t="inlineStr">
         <is>
-          <t>2026-08-27T14:02:13Z</t>
+          <t>2026-08-29T14:28:01Z</t>
         </is>
       </c>
       <c r="F13" s="247" t="inlineStr">
         <is>
-          <t>1A4120300004532000001448</t>
+          <t>1A4120300004532000001528</t>
         </is>
       </c>
       <c r="G13" s="247" t="inlineStr">
@@ -4772,7 +4772,7 @@
       </c>
       <c r="H13" s="262" t="inlineStr">
         <is>
-          <t>[{"Label":"1A4120300004532000001448","Quantity":0,"UnitOfMeasure":"Grams","AdjustmentReason":"Drying","AdjustmentDate":"2026-08-27","ReasonNote":"Evaluation step — adjusting to zero."}]</t>
+          <t>[{"Label":"1A4120300004532000001528","Quantity":0,"UnitOfMeasure":"Grams","AdjustmentReason":"Drying","AdjustmentDate":"2026-08-29","ReasonNote":"Evaluation step — adjusting to zero."}]</t>
         </is>
       </c>
     </row>
@@ -4837,12 +4837,12 @@
       </c>
       <c r="E17" s="250" t="inlineStr">
         <is>
-          <t>2026-08-27T14:02:13Z</t>
+          <t>2026-08-29T14:28:01Z</t>
         </is>
       </c>
       <c r="F17" s="247" t="inlineStr">
         <is>
-          <t>1A4120300004532000001448</t>
+          <t>1A4120300004532000001528</t>
         </is>
       </c>
       <c r="G17" s="247" t="inlineStr">
@@ -4852,7 +4852,7 @@
       </c>
       <c r="H17" s="262" t="inlineStr">
         <is>
-          <t>[{"Label":"1A4120300004532000001448","ActualDate":"2026-08-27"}]</t>
+          <t>[{"Label":"1A4120300004532000001528","ActualDate":"2026-08-29"}]</t>
         </is>
       </c>
     </row>
@@ -4917,12 +4917,12 @@
       </c>
       <c r="E21" s="250" t="inlineStr">
         <is>
-          <t>2026-08-27T14:02:13Z</t>
+          <t>2026-08-29T14:28:01Z</t>
         </is>
       </c>
       <c r="F21" s="247" t="inlineStr">
         <is>
-          <t>1A4120300004532000001448</t>
+          <t>1A4120300004532000001528</t>
         </is>
       </c>
       <c r="G21" s="247" t="inlineStr">
@@ -4932,7 +4932,7 @@
       </c>
       <c r="H21" s="262" t="inlineStr">
         <is>
-          <t>[{"Label":"1A4120300004532000001448"}]</t>
+          <t>[{"Label":"1A4120300004532000001528"}]</t>
         </is>
       </c>
     </row>
@@ -7470,27 +7470,27 @@
       </c>
       <c r="C5" s="248" t="inlineStr">
         <is>
-          <t>SF-SBX-NY-17-30301</t>
+          <t>SF-SBX-NY-5-30301</t>
         </is>
       </c>
       <c r="D5" s="248" t="inlineStr">
         <is>
-          <t>218855</t>
+          <t>218937</t>
         </is>
       </c>
       <c r="E5" s="250" t="inlineStr">
         <is>
-          <t>2026-08-27T13:23:28+00:00</t>
+          <t>2026-08-29T14:28:07+00:00</t>
         </is>
       </c>
       <c r="F5" s="247" t="inlineStr">
         <is>
-          <t>1A4120300004532000001111</t>
+          <t>1A4120300004533000000013</t>
         </is>
       </c>
       <c r="G5" s="247" t="inlineStr">
         <is>
-          <t>https://sandbox-api-ny.metrc.com/labtests/v2/results?packageId=218855&amp;licenseNumber=SF-SBX-NY-17-30301</t>
+          <t>https://sandbox-api-ny.metrc.com/labtests/v2/results?packageId=218937&amp;licenseNumber=SF-SBX-NY-5-30301</t>
         </is>
       </c>
       <c r="H5" s="262" t="inlineStr">
@@ -8196,17 +8196,17 @@
       </c>
       <c r="D5" s="248" t="inlineStr">
         <is>
-          <t>682</t>
+          <t>683</t>
         </is>
       </c>
       <c r="E5" s="250" t="inlineStr">
         <is>
-          <t>2026-08-27T14:02:15Z</t>
+          <t>2026-08-29T14:28:03Z</t>
         </is>
       </c>
       <c r="F5" s="247" t="inlineStr">
         <is>
-          <t>1A4120300004533000000001</t>
+          <t>1A4120300004533000000011</t>
         </is>
       </c>
       <c r="G5" s="248" t="inlineStr">
@@ -8216,7 +8216,7 @@
       </c>
       <c r="H5" s="262" t="inlineStr">
         <is>
-          <t>[{"SalesDateTime":"2026-08-27T14:02:14Z","ExternalReceiptNumber":"TP-0827-1402","SalesCustomerType":"Consumer","PatientLicenseNumber":null,"CaregiverLicenseNumber":null,"IdentificationMethod":null,"PatientRegistrationLocationId":null,"Transactions":[{"PackageLabel":"1A4120300004533000000001","Quantity":1.0,"UnitOfMeasure":"Each","TotalAmount":9.99}]}]</t>
+          <t>[{"SalesDateTime":"2026-08-29T14:28:02Z","ExternalReceiptNumber":"TP-0829-1427","SalesCustomerType":"Consumer","PatientLicenseNumber":null,"CaregiverLicenseNumber":null,"IdentificationMethod":null,"PatientRegistrationLocationId":null,"Transactions":[{"PackageLabel":"1A4120300004533000000011","Quantity":1.0,"UnitOfMeasure":"Each","TotalAmount":9.99}]}]</t>
         </is>
       </c>
     </row>
@@ -8275,17 +8275,17 @@
       </c>
       <c r="D9" s="248" t="inlineStr">
         <is>
-          <t>682</t>
+          <t>683</t>
         </is>
       </c>
       <c r="E9" s="250" t="inlineStr">
         <is>
-          <t>2026-08-27T14:02:15Z</t>
+          <t>2026-08-29T14:28:03Z</t>
         </is>
       </c>
       <c r="F9" s="247" t="inlineStr">
         <is>
-          <t>1A4120300004533000000001</t>
+          <t>1A4120300004533000000011</t>
         </is>
       </c>
       <c r="G9" s="248" t="inlineStr">
@@ -8295,7 +8295,7 @@
       </c>
       <c r="H9" s="262" t="inlineStr">
         <is>
-          <t>[{"SalesDateTime":"2026-08-27T14:02:15Z","ExternalReceiptNumber":"TP-0827-1402","SalesCustomerType":"Consumer","PatientLicenseNumber":null,"CaregiverLicenseNumber":null,"IdentificationMethod":null,"PatientRegistrationLocationId":null,"Transactions":[{"PackageLabel":"1A4120300004533000000001","Quantity":2.0,"UnitOfMeasure":"Each","TotalAmount":19.98}],"Id":682}]</t>
+          <t>[{"SalesDateTime":"2026-08-29T14:28:03Z","ExternalReceiptNumber":"TP-0829-1427","SalesCustomerType":"Consumer","PatientLicenseNumber":null,"CaregiverLicenseNumber":null,"IdentificationMethod":null,"PatientRegistrationLocationId":null,"Transactions":[{"PackageLabel":"1A4120300004533000000011","Quantity":2.0,"UnitOfMeasure":"Each","TotalAmount":19.98}],"Id":683}]</t>
         </is>
       </c>
     </row>
@@ -8348,22 +8348,22 @@
       </c>
       <c r="D13" s="248" t="inlineStr">
         <is>
-          <t>682</t>
+          <t>683</t>
         </is>
       </c>
       <c r="E13" s="250" t="inlineStr">
         <is>
-          <t>2026-08-27T14:02:15Z</t>
+          <t>2026-08-29T14:28:04Z</t>
         </is>
       </c>
       <c r="F13" s="247" t="inlineStr">
         <is>
-          <t>1A4120300004533000000001</t>
+          <t>1A4120300004533000000011</t>
         </is>
       </c>
       <c r="G13" s="248" t="inlineStr">
         <is>
-          <t>https://sandbox-api-ny.metrc.com/sales/v2/receipts/682?licenseNumber=SF-SBX-NY-5-30301</t>
+          <t>https://sandbox-api-ny.metrc.com/sales/v2/receipts/683?licenseNumber=SF-SBX-NY-5-30301</t>
         </is>
       </c>
       <c r="H13" s="248" t="inlineStr">
@@ -8433,7 +8433,7 @@
       </c>
       <c r="E17" s="250" t="inlineStr">
         <is>
-          <t>2026-08-27T14:02:15Z</t>
+          <t>2026-08-29T14:28:04Z</t>
         </is>
       </c>
       <c r="F17" s="247" t="inlineStr">
@@ -8501,17 +8501,17 @@
       </c>
       <c r="D21" s="248" t="inlineStr">
         <is>
-          <t>679</t>
+          <t>684</t>
         </is>
       </c>
       <c r="E21" s="250" t="inlineStr">
         <is>
-          <t>2026-08-27T14:02:15Z</t>
+          <t>2026-08-29T14:28:04Z</t>
         </is>
       </c>
       <c r="F21" s="247" t="inlineStr">
         <is>
-          <t>1A4120300004533000000001</t>
+          <t>1A4120300004533000000011</t>
         </is>
       </c>
       <c r="G21" s="248" t="inlineStr">
@@ -8521,7 +8521,7 @@
       </c>
       <c r="H21" s="262" t="inlineStr">
         <is>
-          <t>[{"SalesDateTime":"2026-08-27T14:02:15Z","ExternalReceiptNumber":"TP-0827-1402-EP","SalesCustomerType":"ExternalPatient","PatientLicenseNumber":"PTN-123-456","CaregiverLicenseNumber":null,"IdentificationMethod":null,"PatientRegistrationLocationId":null,"Transactions":[{"PackageLabel":"1A4120300004533000000001","Quantity":1.0,"UnitOfMeasure":"Each","TotalAmount":9.99}]}]</t>
+          <t>[{"SalesDateTime":"2026-08-29T14:28:04Z","ExternalReceiptNumber":"TP-0829-1427-EP","SalesCustomerType":"ExternalPatient","PatientLicenseNumber":"PTN-123-456","CaregiverLicenseNumber":null,"IdentificationMethod":null,"PatientRegistrationLocationId":null,"Transactions":[{"PackageLabel":"1A4120300004533000000011","Quantity":1.0,"UnitOfMeasure":"Each","TotalAmount":9.99}]}]</t>
         </is>
       </c>
     </row>
@@ -8857,17 +8857,17 @@
       </c>
       <c r="D5" s="248" t="inlineStr">
         <is>
-          <t>405</t>
+          <t>411</t>
         </is>
       </c>
       <c r="E5" s="250" t="inlineStr">
         <is>
-          <t>2026-08-27T14:02:16Z</t>
+          <t>2026-08-29T14:28:05Z</t>
         </is>
       </c>
       <c r="F5" s="247" t="inlineStr">
         <is>
-          <t>1A4120300004533000000002</t>
+          <t>1A4120300004533000000012</t>
         </is>
       </c>
       <c r="G5" s="247" t="inlineStr">
@@ -8877,7 +8877,7 @@
       </c>
       <c r="H5" s="262" t="inlineStr">
         <is>
-          <t>[{"SalesDateTime":"2026-08-27T14:02:15Z","SalesCustomerType":"Consumer","PatientLicenseNumber":null,"ConsumerId":null,"DriverEmployeeId":"1","DriverName":"Evaluation Driver","DriversLicenseNumber":"D0000001","PhoneNumberForQuestions":"+1-555-000-0000","VehicleMake":"Car","VehicleModel":"Small","VehicleLicensePlateNumber":"TP-0001","RecipientAddressStreet1":"1 Evaluation Way","RecipientAddressCity":"Albany","RecipientAddressState":"NY","RecipientAddressPostalCode":"12207","PlannedRoute":"Drive to destination.","EstimatedDepartureDateTime":"2026-08-27T15:02:15Z","EstimatedArrivalDateTime":"2026-08-27T17:02:15Z","Transactions":[{"PackageLabel":"1A4120300004533000000002","Quantity":1.0,"UnitOfMeasure":"Each","TotalAmount":9.99},{"PackageLabel":"1A4120300004533000000003","Quantity":1.0,"UnitOfMeasure":"Each","TotalAmount":19.98},{"PackageLabel":"1A4120300004533000000004","Quantity":1.0,"UnitOfMeasure":"Each","TotalAmount":29.97}]}]</t>
+          <t>[{"SalesDateTime":"2026-08-29T14:28:04Z","SalesCustomerType":"Consumer","PatientLicenseNumber":null,"ConsumerId":null,"DriverEmployeeId":"1","DriverName":"Evaluation Driver","DriversLicenseNumber":"D0000001","PhoneNumberForQuestions":"+1-555-000-0000","VehicleMake":"Car","VehicleModel":"Small","VehicleLicensePlateNumber":"TP-0001","RecipientAddressStreet1":"1 Evaluation Way","RecipientAddressCity":"Albany","RecipientAddressState":"NY","RecipientAddressPostalCode":"12207","PlannedRoute":"Drive to destination.","EstimatedDepartureDateTime":"2026-08-29T15:28:04Z","EstimatedArrivalDateTime":"2026-08-29T17:28:04Z","Transactions":[{"PackageLabel":"1A4120300004533000000012","Quantity":1.0,"UnitOfMeasure":"Each","TotalAmount":9.99},{"PackageLabel":"1A4120300004533000000013","Quantity":1.0,"UnitOfMeasure":"Each","TotalAmount":19.98},{"PackageLabel":"1A4120300004533000000014","Quantity":1.0,"UnitOfMeasure":"Each","TotalAmount":29.97}]}]</t>
         </is>
       </c>
     </row>
@@ -8937,17 +8937,17 @@
       </c>
       <c r="D9" s="248" t="inlineStr">
         <is>
-          <t>405</t>
+          <t>411</t>
         </is>
       </c>
       <c r="E9" s="250" t="inlineStr">
         <is>
-          <t>2026-08-27T14:02:16Z</t>
+          <t>2026-08-29T14:28:05Z</t>
         </is>
       </c>
       <c r="F9" s="247" t="inlineStr">
         <is>
-          <t>1A4120300004533000000002</t>
+          <t>1A4120300004533000000012</t>
         </is>
       </c>
       <c r="G9" s="247" t="inlineStr">
@@ -8957,7 +8957,7 @@
       </c>
       <c r="H9" s="262" t="inlineStr">
         <is>
-          <t>[{"SalesDateTime":"2026-08-27T14:02:15Z","SalesCustomerType":"Consumer","PatientLicenseNumber":null,"ConsumerId":null,"DriverEmployeeId":"1","DriverName":"Evaluation Driver","DriversLicenseNumber":"D0000001","PhoneNumberForQuestions":"+1-555-000-0000","VehicleMake":"Car","VehicleModel":"Small","VehicleLicensePlateNumber":"TP-0001","RecipientAddressStreet1":"1 Evaluation Way","RecipientAddressCity":"Albany","RecipientAddressState":"NY","RecipientAddressPostalCode":"12207","PlannedRoute":"Drive to destination.","EstimatedDepartureDateTime":"2026-08-27T15:02:15Z","EstimatedArrivalDateTime":"2026-08-27T17:02:15Z","Transactions":[{"PackageLabel":"1A4120300004533000000002","Quantity":1.0,"UnitOfMeasure":"Each","TotalAmount":9.99},{"PackageLabel":"1A4120300004533000000003","Quantity":1.0,"UnitOfMeasure":"Each","TotalAmount":19.98}],"Id":405}]</t>
+          <t>[{"SalesDateTime":"2026-08-29T14:28:04Z","SalesCustomerType":"Consumer","PatientLicenseNumber":null,"ConsumerId":null,"DriverEmployeeId":"1","DriverName":"Evaluation Driver","DriversLicenseNumber":"D0000001","PhoneNumberForQuestions":"+1-555-000-0000","VehicleMake":"Car","VehicleModel":"Small","VehicleLicensePlateNumber":"TP-0001","RecipientAddressStreet1":"1 Evaluation Way","RecipientAddressCity":"Albany","RecipientAddressState":"NY","RecipientAddressPostalCode":"12207","PlannedRoute":"Drive to destination.","EstimatedDepartureDateTime":"2026-08-29T15:28:04Z","EstimatedArrivalDateTime":"2026-08-29T17:28:04Z","Transactions":[{"PackageLabel":"1A4120300004533000000012","Quantity":1.0,"UnitOfMeasure":"Each","TotalAmount":9.99},{"PackageLabel":"1A4120300004533000000013","Quantity":1.0,"UnitOfMeasure":"Each","TotalAmount":19.98}],"Id":411}]</t>
         </is>
       </c>
     </row>
@@ -9010,17 +9010,17 @@
       </c>
       <c r="D13" s="248" t="inlineStr">
         <is>
-          <t>405</t>
+          <t>411</t>
         </is>
       </c>
       <c r="E13" s="250" t="inlineStr">
         <is>
-          <t>2026-08-27T14:02:16Z</t>
+          <t>2026-08-29T14:28:06Z</t>
         </is>
       </c>
       <c r="F13" s="247" t="inlineStr">
         <is>
-          <t>1A4120300004533000000002</t>
+          <t>1A4120300004533000000012</t>
         </is>
       </c>
       <c r="G13" s="247" t="inlineStr">
@@ -9030,7 +9030,7 @@
       </c>
       <c r="H13" s="262" t="inlineStr">
         <is>
-          <t>[{"Id":405,"ActualArrivalDateTime":"2026-08-27T14:02:16Z","PaymentType":null,"AcceptedPackages":["1A4120300004533000000002"],"ReturnedPackages":[{"Label":"1A4120300004533000000003","ReturnQuantityVerified":1.0,"ReturnUnitOfMeasure":"Each","ReturnReason":"Unable to Deliver","ReturnReasonNote":"Evaluation step"}]}]</t>
+          <t>[{"Id":411,"ActualArrivalDateTime":"2026-08-29T14:28:05Z","PaymentType":null,"AcceptedPackages":["1A4120300004533000000012"],"ReturnedPackages":[{"Label":"1A4120300004533000000013","ReturnQuantityVerified":1.0,"ReturnUnitOfMeasure":"Each","ReturnReason":"Unable to Deliver","ReturnReasonNote":"Evaluation step"}]}]</t>
         </is>
       </c>
     </row>
@@ -10364,7 +10364,7 @@
       </c>
       <c r="G5" s="247" t="inlineStr">
         <is>
-          <t>https://sandbox-api-ny.metrc.com/transfers/v2/incoming?lastModifiedStart=2026-08-26T14%3A02%3A32Z&amp;lastModifiedEnd=2026-08-27T14%3A02%3A32Z&amp;licenseNumber=SF-SBX-NY-14-30301</t>
+          <t>https://sandbox-api-ny.metrc.com/transfers/v2/incoming?lastModifiedStart=2026-08-26T14%3A28%3A26Z&amp;lastModifiedEnd=2026-08-27T14%3A28%3A26Z&amp;licenseNumber=SF-SBX-NY-14-30301</t>
         </is>
       </c>
       <c r="H5" s="262" t="inlineStr">
@@ -10438,7 +10438,7 @@
       </c>
       <c r="G9" s="247" t="inlineStr">
         <is>
-          <t>https://sandbox-api-ny.metrc.com/transfers/v2/outgoing?lastModifiedStart=2026-08-26T14%3A02%3A32Z&amp;lastModifiedEnd=2026-08-27T14%3A02%3A32Z&amp;licenseNumber=SF-SBX-NY-3-30301</t>
+          <t>https://sandbox-api-ny.metrc.com/transfers/v2/outgoing?lastModifiedStart=2026-08-26T14%3A28%3A28Z&amp;lastModifiedEnd=2026-08-27T14%3A28%3A28Z&amp;licenseNumber=SF-SBX-NY-3-30301</t>
         </is>
       </c>
       <c r="H9" s="262" t="inlineStr">
@@ -10511,7 +10511,7 @@
       </c>
       <c r="G13" s="247" t="inlineStr">
         <is>
-          <t>https://sandbox-api-ny.metrc.com/transfers/v2/rejected?lastModifiedStart=2026-08-25T14%3A02%3A33Z&amp;lastModifiedEnd=2026-08-26T14%3A02%3A33Z&amp;licenseNumber=SF-SBX-NY-3-30301</t>
+          <t>https://sandbox-api-ny.metrc.com/transfers/v2/rejected?lastModifiedStart=2026-08-27T14%3A28%3A29Z&amp;lastModifiedEnd=2026-08-28T14%3A28%3A29Z&amp;licenseNumber=SF-SBX-NY-3-30301</t>
         </is>
       </c>
       <c r="H13" s="262" t="inlineStr">
@@ -10661,7 +10661,7 @@
       </c>
       <c r="E21" s="250" t="inlineStr">
         <is>
-          <t>2026-08-27T14:02:33Z</t>
+          <t>2026-08-29T14:28:29Z</t>
         </is>
       </c>
       <c r="F21" s="247" t="inlineStr">
@@ -10741,7 +10741,7 @@
       </c>
       <c r="E25" s="250" t="inlineStr">
         <is>
-          <t>2026-08-27T14:02:33Z</t>
+          <t>2026-08-29T14:28:29Z</t>
         </is>
       </c>
       <c r="F25" s="247" t="inlineStr">
@@ -11145,12 +11145,12 @@
       </c>
       <c r="D5" s="248" t="inlineStr">
         <is>
-          <t>15910</t>
+          <t>16009</t>
         </is>
       </c>
       <c r="E5" s="250" t="inlineStr">
         <is>
-          <t>2026-08-29T13:32:25Z</t>
+          <t>2026-08-29T14:28:06Z</t>
         </is>
       </c>
       <c r="F5" s="247" t="inlineStr">
@@ -11165,7 +11165,7 @@
       </c>
       <c r="H5" s="262" t="inlineStr">
         <is>
-          <t>[{"Name":"TP Template A 0829-1332","TransporterFacilityLicenseNumber":null,"DriverOccupationalLicenseNumber":null,"DriverName":null,"DriverLicenseNumber":null,"PhoneNumberForQuestions":null,"VehicleMake":null,"VehicleModel":null,"VehicleLicensePlateNumber":null,"VehicleRegistrationNumber":null,"Destinations":[{"RecipientLicenseNumber":"SF-SBX-NY-6-13402","InvoiceNumber":"INV-A-0829-1332","TransferTypeName":"Unaffiliated Transfer","PlannedRoute":"Evaluation route.","EstimatedDepartureDateTime":"2026-08-29T14:32:24Z","EstimatedArrivalDateTime":"2026-08-29T17:32:24Z","Transporters":[],"Packages":[]}]}]</t>
+          <t>[{"Name":"TP Template A 0829-1427","TransporterFacilityLicenseNumber":null,"DriverOccupationalLicenseNumber":null,"DriverName":null,"DriverLicenseNumber":null,"PhoneNumberForQuestions":null,"VehicleMake":null,"VehicleModel":null,"VehicleLicensePlateNumber":null,"VehicleRegistrationNumber":null,"Destinations":[{"RecipientLicenseNumber":"SF-SBX-NY-6-13402","InvoiceNumber":"INV-A-0829-1427","TransferTypeName":"Unaffiliated Transfer","PlannedRoute":"Evaluation route.","EstimatedDepartureDateTime":"2026-08-29T15:28:06Z","EstimatedArrivalDateTime":"2026-08-29T18:28:06Z","Transporters":[],"Packages":[]}]}]</t>
         </is>
       </c>
     </row>
@@ -11219,12 +11219,12 @@
       </c>
       <c r="D9" s="248" t="inlineStr">
         <is>
-          <t>15911</t>
+          <t>16010</t>
         </is>
       </c>
       <c r="E9" s="250" t="inlineStr">
         <is>
-          <t>2026-08-29T13:32:25Z</t>
+          <t>2026-08-29T14:28:07Z</t>
         </is>
       </c>
       <c r="F9" s="247" t="inlineStr">
@@ -11239,7 +11239,7 @@
       </c>
       <c r="H9" s="262" t="inlineStr">
         <is>
-          <t>[{"Name":"TP Template B 0829-1332","TransporterFacilityLicenseNumber":null,"DriverOccupationalLicenseNumber":null,"DriverName":null,"DriverLicenseNumber":null,"PhoneNumberForQuestions":null,"VehicleMake":null,"VehicleModel":null,"VehicleLicensePlateNumber":null,"VehicleRegistrationNumber":null,"Destinations":[{"RecipientLicenseNumber":"SF-SBX-NY-6-13402","InvoiceNumber":"INV-B-0829-1332","TransferTypeName":"Unaffiliated Transfer","PlannedRoute":"Evaluation route.","EstimatedDepartureDateTime":"2026-08-29T14:32:24Z","EstimatedArrivalDateTime":"2026-08-29T17:32:24Z","Transporters":[],"Packages":[]}]}]</t>
+          <t>[{"Name":"TP Template B 0829-1427","TransporterFacilityLicenseNumber":null,"DriverOccupationalLicenseNumber":null,"DriverName":null,"DriverLicenseNumber":null,"PhoneNumberForQuestions":null,"VehicleMake":null,"VehicleModel":null,"VehicleLicensePlateNumber":null,"VehicleRegistrationNumber":null,"Destinations":[{"RecipientLicenseNumber":"SF-SBX-NY-6-13402","InvoiceNumber":"INV-B-0829-1427","TransferTypeName":"Unaffiliated Transfer","PlannedRoute":"Evaluation route.","EstimatedDepartureDateTime":"2026-08-29T15:28:06Z","EstimatedArrivalDateTime":"2026-08-29T18:28:06Z","Transporters":[],"Packages":[]}]}]</t>
         </is>
       </c>
     </row>
@@ -11292,12 +11292,12 @@
       </c>
       <c r="D13" s="248" t="inlineStr">
         <is>
-          <t>15910, 15911</t>
+          <t>16009, 16010</t>
         </is>
       </c>
       <c r="E13" s="250" t="inlineStr">
         <is>
-          <t>2026-08-29T13:32:25+00:00</t>
+          <t>2026-08-29T14:28:07+00:00</t>
         </is>
       </c>
       <c r="F13" s="247" t="inlineStr">
@@ -11307,12 +11307,12 @@
       </c>
       <c r="G13" s="247" t="inlineStr">
         <is>
-          <t>https://sandbox-api-ny.metrc.com/transfers/v2/templates/outgoing?lastModifiedStart=2026-08-28T13%3A32%3A25Z&amp;lastModifiedEnd=2026-08-29T13%3A32%3A25Z&amp;licenseNumber=SF-SBX-NY-3-30301</t>
+          <t>https://sandbox-api-ny.metrc.com/transfers/v2/templates/outgoing?lastModifiedStart=2026-08-28T14%3A28%3A07Z&amp;lastModifiedEnd=2026-08-29T14%3A28%3A07Z&amp;licenseNumber=SF-SBX-NY-3-30301</t>
         </is>
       </c>
       <c r="H13" s="262" t="inlineStr">
         <is>
-          <t>{"Data":[{"Id":15910,"ManifestNumber":"T-0000015910","InvoiceNumber":"INV-A-0829-1332","ShipmentLicenseType":"Licensed","ShipperFacilityLicenseNumber":"SF-SBX-NY-3-30301","ShipperFacilityName":"Sandbox AU Cultivator","Name":"TP Template A 0829-1332","TransporterFacilityLicenseNumber":null,"TransporterFacilityName":null,"DriverName":null,"DriverOccupationalLicenseNumber":null,"DriverVehicleLicenseNumber":null,"VehicleMake":null,"VehicleModel":null,"VehicleLicensePlateNumber":null,"VehicleRegistrationNumber":null,"DeliveryCount":1,"ReceivedDeliveryCount":0,"PackageCount":0,"ReceivedPackageCount":0,"ContainsPlantPackage":false,"ContainsProductPackage":false,"ContainsTradeSample":false,"ContainsDonation":false,"ContainsTestingSample":false,"ContainsProductRequiresRemediation":false,"ContainsRemediatedProductPackage":false,"ContainsPreTreatedProductPackage":false,"IsVoided":false,"CreatedDateTime":"2026-08-29T13:32:25+00:00","CreatedByUserName":"Pablo Dayton","LastModified":"2026-08-29T13:32:25+00:00","DeliveryId":0,"RecipientFacilityLicenseNumber":null,"RecipientFacilityName":null,"ShipmentTypeName":null,"ShipmentTransactionType":null,"EstimatedDepartureDateTime":"0001-01-01T00:00:00.000","ActualDepartureDateTime":null,"EstimatedArrivalDateTime":"0001-01-01T00:00:00.000","ActualArrivalDateTime":null,"DeliveryPackageCount":0,"DeliveryReceivedPackageCount":0,"ReceivedDateTime":null,"EstimatedReturnDepartureDateTime":null,"ActualReturnDepartureDateTime":null,"EstimatedReturnArrivalDateTime":null,"ActualReturnArrivalDateTime":null,"OriginatingTemplateId":null},{"Id":15911,"ManifestNumber":"T-0000015911","InvoiceNumber":"INV-B-0829-1332","ShipmentLicenseType":"Licensed","ShipperFacilityLicenseNumber":"SF-SBX-NY-3-30301","ShipperFacilityName":"Sandbox AU Cultivator","Name":"TP Template B 0829-1332","TransporterFacilityLicenseNumber":null,"TransporterFacilityName":null,"DriverName":null,"DriverOccupationalLicenseNumber":null,"DriverVehicleLicenseNumber":null,"VehicleMake":null,"VehicleModel":null,"VehicleLicensePlateNumber":null,"VehicleRegistrationNumber":null,"DeliveryCount":1,"ReceivedDeliveryCount":0,"PackageCount":0,"ReceivedPackageCount":0,"ContainsPlantPackage":false,"ContainsProductPackage":false,"ContainsTradeSample":false,"ContainsDonation":false,"ContainsTestingSample":false,"ContainsProductRequiresRemediation":false,"ContainsRemediatedProductPackage":false,"ContainsPreTreatedProductPackage":false,"IsVoided":false,"CreatedDateTime":"2026-08-29T13:32:25+00:00","CreatedByUserName":"Pablo Dayton","LastModified":"2026-08-29T13:32:25+00:00","DeliveryId":0,"RecipientFacilityLicenseNumber":null,"RecipientFacilityName":null,"ShipmentTypeName":null,"ShipmentTransactionType":null,"EstimatedDepartureDateTime":"0001-01-01T00:00:00.000","ActualDepartureDateTime":null,"EstimatedArrivalDateTime":"0001-01-01T00:00:00.000","ActualArrivalDateTime":null,"DeliveryPackageCount":0,"DeliveryReceivedPackageCount":0,"ReceivedDateTime":null,"EstimatedReturnDepartureDateTime":null,"ActualReturnDepartureDateTime":null,"EstimatedReturnArrivalDateTime":null,"ActualReturnArrivalDateTime":null,"OriginatingTemplateId":null}],"Total":2,"TotalRecords":2,"PageSize":2,"RecordsOnPage":2,"Page":1,"CurrentPage":1,"TotalPages":1}</t>
+          <t>{"Data":[{"Id":16009,"ManifestNumber":"T-0000016009","InvoiceNumber":"INV-A-0829-1427","ShipmentLicenseType":"Licensed","ShipperFacilityLicenseNumber":"SF-SBX-NY-3-30301","ShipperFacilityName":"Sandbox AU Cultivator","Name":"TP Template A 0829-1427","TransporterFacilityLicenseNumber":null,"TransporterFacilityName":null,"DriverName":null,"DriverOccupationalLicenseNumber":null,"DriverVehicleLicenseNumber":null,"VehicleMake":null,"VehicleModel":null,"VehicleLicensePlateNumber":null,"VehicleRegistrationNumber":null,"DeliveryCount":1,"ReceivedDeliveryCount":0,"PackageCount":0,"ReceivedPackageCount":0,"ContainsPlantPackage":false,"ContainsProductPackage":false,"ContainsTradeSample":false,"ContainsDonation":false,"ContainsTestingSample":false,"ContainsProductRequiresRemediation":false,"ContainsRemediatedProductPackage":false,"ContainsPreTreatedProductPackage":false,"IsVoided":false,"CreatedDateTime":"2026-08-29T14:28:07+00:00","CreatedByUserName":"Pablo Dayton","LastModified":"2026-08-29T14:28:07+00:00","DeliveryId":0,"RecipientFacilityLicenseNumber":null,"RecipientFacilityName":null,"ShipmentTypeName":null,"ShipmentTransactionType":null,"EstimatedDepartureDateTime":"0001-01-01T00:00:00.000","ActualDepartureDateTime":null,"EstimatedArrivalDateTime":"0001-01-01T00:00:00.000","ActualArrivalDateTime":null,"DeliveryPackageCount":0,"DeliveryReceivedPackageCount":0,"ReceivedDateTime":null,"EstimatedReturnDepartureDateTime":null,"ActualReturnDepartureDateTime":null,"EstimatedReturnArrivalDateTime":null,"ActualReturnArrivalDateTime":null,"OriginatingTemplateId":null},{"Id":16010,"ManifestNumber":"T-0000016010","InvoiceNumber":"INV-B-0829-1427","ShipmentLicenseType":"Licensed","ShipperFacilityLicenseNumber":"SF-SBX-NY-3-30301","ShipperFacilityName":"Sandbox AU Cultivator","Name":"TP Template B 0829-1427","TransporterFacilityLicenseNumber":null,"TransporterFacilityName":null,"DriverName":null,"DriverOccupationalLicenseNumber":null,"DriverVehicleLicenseNumber":null,"VehicleMake":null,"VehicleModel":null,"VehicleLicensePlateNumber":null,"VehicleRegistrationNumber":null,"DeliveryCount":1,"ReceivedDeliveryCount":0,"PackageCount":0,"ReceivedPackageCount":0,"ContainsPlantPackage":false,"ContainsProductPackage":false,"ContainsTradeSample":false,"ContainsDonation":false,"ContainsTestingSample":false,"ContainsProductRequiresRemediation":false,"ContainsRemediatedProductPackage":false,"ContainsPreTreatedProductPackage":false,"IsVoided":false,"CreatedDateTime":"2026-08-29T14:28:07+00:00","CreatedByUserName":"Pablo Dayton","LastModified":"2026-08-29T14:28:07+00:00","DeliveryId":0,"RecipientFacilityLicenseNumber":null,"RecipientFacilityName":null,"ShipmentTypeName":null,"ShipmentTransactionType":null,"EstimatedDepartureDateTime":"0001-01-01T00:00:00.000","ActualDepartureDateTime":null,"EstimatedArrivalDateTime":"0001-01-01T00:00:00.000","ActualArrivalDateTime":null,"DeliveryPackageCount":0,"DeliveryReceivedPackageCount":0,"ReceivedDateTime":null,"EstimatedReturnDepartureDateTime":null,"ActualReturnDepartureDateTime":null,"EstimatedReturnArrivalDateTime":null,"ActualReturnArrivalDateTime":null,"OriginatingTemplateId":null},{"Id":15912,"ManifestNumber":"T-0000015912","InvoiceNumber":"INV-B-0829-1426","ShipmentLicenseType":"Licensed","ShipperFacilityLicenseNumber":"SF-SBX-NY-3-30301","ShipperFacilityName":"Sandbox AU Cultivator","Name":"TP Template B 0829-1426","TransporterFacilityLicenseNumber":null,"TransporterFacilityName":null,"DriverName":null,"DriverOccupationalLicenseNumber":null,"DriverVehicleLicenseNumber":null,"VehicleMake":null,"VehicleModel":null,"VehicleLicensePlateNumber":null,"VehicleRegistrationNumber":null,"DeliveryCount":1,"ReceivedDeliveryCount":0,"PackageCount":0,"ReceivedPackageCount":0,"ContainsPlantPackage":false,"ContainsProductPackage":false,"ContainsTradeSample":false,"ContainsDonation":false,"ContainsTestingSample":false,"ContainsProductRequiresRemediation":false,"ContainsRemediatedProductPackage":false,"ContainsPreTreatedProductPackage":false,"IsVoided":false,"CreatedDateTime":"2026-08-29T14:26:36+00:00","CreatedByUserName":"Pablo Dayton","LastModified":"2026-08-29T14:26:36+00:00","DeliveryId":0,"RecipientFacilityLicenseNumber":null,"RecipientFacilityName":null,"ShipmentTypeName":null,"ShipmentTransactionType":null,"EstimatedDepartureDateTime":"0001-01-01T00:00:00.000","ActualDepartureDateTime":null,"EstimatedArrivalDateTime":"0001-01-01T00:00:00.000","ActualArrivalDateTime":null,"DeliveryPackageCount":0,"DeliveryReceivedPackageCount":0,"ReceivedDateTime":null,"EstimatedReturnDepartureDateTime":null,"ActualReturnDepartureDateTime":null,"EstimatedReturnArrivalDateTime":null,"ActualReturnArrivalDateTime":null,"OriginatingTemplateId":null},{"Id":16008,"ManifestNumber":"T-0000016008","InvoiceNumber":"INV-A-0829-1426","ShipmentLicenseType":"Licensed","ShipperFacilityLicenseNumber":"SF-SBX-NY-3-30301","ShipperFacilityName":"Sandbox AU Cultivator","Name":"TP Template A 0829-1426 (Updated)","TransporterFacilityLicenseNumber":null,"TransporterFacilityName":null,"DriverName":null,"DriverOccupationalLicenseNumber":null,"DriverVehicleLicenseNumber":null,"VehicleMake":null,"VehicleModel":null,"VehicleLicensePlateNumber":null,"VehicleRegistrationNumber":null,"DeliveryCount":1,"ReceivedDeliveryCount":0,"PackageCount":0,"ReceivedPackageCount":0,"ContainsPlantPackage":false,"ContainsProductPackage":false,"ContainsTradeSample":false,"ContainsDonation":false,"ContainsTestingSample":false,"ContainsProductRequiresRemediation":false,"ContainsRemediatedProductPackage":false,"ContainsPreTreatedProductPackage":false,"IsVoided":false,"CreatedDateTime":"2026-08-29T14:26:36+00:00","CreatedByUserName":"Pablo Dayton","LastModified":"2026-08-29T14:26:36+00:00","DeliveryId":0,"RecipientFacilityLicenseNumber":null,"RecipientFacilityName":null,"ShipmentTypeName":null,"ShipmentTransactionType":null,"EstimatedDepartureDateTime":"0001-01-01T00:00:00.000","ActualDepartureDateTime":null,"EstimatedArrivalDateTime":"0001-01-01T00:00:00.000","ActualArrivalDateTime":null,"DeliveryPackageCount":0,"DeliveryReceivedPackageCount":0,"ReceivedDateTime":null,"EstimatedReturnDepartureDateTime":null,"ActualReturnDepartureDateTime":null,"EstimatedReturnArrivalDateTime":null,"ActualReturnArrivalDateTime":null,"OriginatingTemplateId":null},{"Id":15910,"ManifestNumber":"T-0000015910","InvoiceNumber":"INV-A-0829-1332","ShipmentLicenseType":"Licensed","ShipperFacilityLicenseNumber":"SF-SBX-NY-3-30301","ShipperFacilityName":"Sandbox AU Cultivator","Name":"TP Template A 0829-1332 (Updated)","TransporterFacilityLicenseNumber":null,"TransporterFacilityName":null,"DriverName":null,"DriverOccupationalLicenseNumber":null,"DriverVehicleLicenseNumber":null,"VehicleMake":null,"VehicleModel":null,"VehicleLicensePlateNumber":null,"VehicleRegistrationNumber":null,"DeliveryCount":1,"ReceivedDeliveryCount":0,"PackageCount":0,"ReceivedPackageCount":0,"ContainsPlantPackage":false,"ContainsProductPackage":false,"ContainsTradeSample":false,"ContainsDonation":false,"ContainsTestingSample":false,"ContainsProductRequiresRemediation":false,"ContainsRemediatedProductPackage":false,"ContainsPreTreatedProductPackage":false,"IsVoided":false,"CreatedDateTime":"2026-08-29T13:32:25+00:00","CreatedByUserName":"Pablo Dayton","LastModified":"2026-08-29T13:32:26+00:00","DeliveryId":0,"RecipientFacilityLicenseNumber":null,"RecipientFacilityName":null,"ShipmentTypeName":null,"ShipmentTransactionType":null,"EstimatedDepartureDateTime":"0001-01-01T00:00:00.000","ActualDepartureDateTime":null,"EstimatedArrivalDateTime":"0001-01-01T00:00:00.000","ActualArrivalDateTime":null,"DeliveryPackageCount":0,"DeliveryReceivedPackageCount":0,"ReceivedDateTime":null,"EstimatedReturnDepartureDateTime":null,"ActualReturnDepartureDateTime":null,"EstimatedReturnArrivalDateTime":null,"ActualReturnArrivalDateTime":null,"OriginatingTemplateId":null},{"Id":15911,"ManifestNumber":"T-0000015911","InvoiceNumber":"INV-B-0829-1332","ShipmentLicenseType":"Licensed","ShipperFacilityLicenseNumber":"SF-SBX-NY-3-30301","ShipperFacilityName":"Sandbox AU Cultivator","Name":"TP Template B 0829-1332","TransporterFacilityLicenseNumber":null,"TransporterFacilityName":null,"DriverName":null,"DriverOccupationalLicenseNumber":null,"DriverVehicleLicenseNumber":null,"VehicleMake":null,"VehicleModel":null,"VehicleLicensePlateNumber":null,"VehicleRegistrationNumber":null,"DeliveryCount":1,"ReceivedDeliveryCount":0,"PackageCount":0,"ReceivedPackageCount":0,"ContainsPlantPackage":false,"ContainsProductPackage":false,"ContainsTradeSample":false,"ContainsDonation":false,"ContainsTestingSample":false,"ContainsProductRequiresRemediation":false,"ContainsRemediatedProductPackage":false,"ContainsPreTreatedProductPackage":false,"IsVoided":false,"CreatedDateTime":"2026-08-29T13:32:25+00:00","CreatedByUserName":"Pablo Dayton","LastModified":"2026-08-29T13:32:25+00:00","DeliveryId":0,"RecipientFacilityLicenseNumber":null,"RecipientFacilityName":null,"ShipmentTypeName":null,"ShipmentTransactionType":null,"EstimatedDepartureDateTime":"0001-01-01T00:00:00.000","ActualDepartureDateTime":null,"EstimatedArrivalDateTime":"0001-01-01T00:00:00.000","ActualArrivalDateTime":null,"DeliveryPackageCount":0,"DeliveryReceivedPackageCount":0,"ReceivedDateTime":null,"EstimatedReturnDepartureDateTime":null,"ActualReturnDepartureDateTime":null,"EstimatedReturnArrivalDateTime":null,"ActualReturnArrivalDateTime":null,"OriginatingTemplateId":null}],"Total":6,"TotalRecords":6,"PageSize":6,"RecordsOnPage":6,"Page":1,"CurrentPage":1,"TotalPages":1}</t>
         </is>
       </c>
     </row>
@@ -11372,12 +11372,12 @@
       </c>
       <c r="D17" s="248" t="inlineStr">
         <is>
-          <t>15910</t>
+          <t>16009</t>
         </is>
       </c>
       <c r="E17" s="250" t="inlineStr">
         <is>
-          <t>2026-08-29T13:32:25Z</t>
+          <t>2026-08-29T14:28:07Z</t>
         </is>
       </c>
       <c r="F17" s="247" t="inlineStr">
@@ -11387,12 +11387,12 @@
       </c>
       <c r="G17" s="247" t="inlineStr">
         <is>
-          <t>https://sandbox-api-ny.metrc.com/transfers/v2/templates/outgoing/15910/deliveries</t>
+          <t>https://sandbox-api-ny.metrc.com/transfers/v2/templates/outgoing/16009/deliveries</t>
         </is>
       </c>
       <c r="H17" s="262" t="inlineStr">
         <is>
-          <t>{"Data":[{"Id":16412,"ManifestNumber":null,"DeliveryNumber":0,"RecipientFacilityLicenseNumber":"SF-SBX-NY-6-13402","RecipientFacilityName":"Sandbox AU Distributor","ShipmentTypeName":"Unaffiliated Transfer","ShipmentTransactionType":"Wholesale","InvoiceNumber":"INV-A-0829-1332","PaymentTermDays":null,"PaymentDueDate":null,"EstimatedDepartureDateTime":"2026-08-29T14:32:00.000","ActualDepartureDateTime":null,"EstimatedArrivalDateTime":"2026-08-29T17:32:00.000","ActualArrivalDateTime":null,"GrossWeight":null,"GrossUnitOfWeightId":null,"GrossUnitOfWeightName":null,"PlannedRoute":"Evaluation route.","DeliveryPackageCount":0,"DeliveryReceivedPackageCount":0,"ReceivedDateTime":null,"EstimatedReturnDepartureDateTime":null,"ActualReturnDepartureDateTime":null,"EstimatedReturnArrivalDateTime":null,"ActualReturnArrivalDateTime":null,"RejectedPackagesReturned":false,"PDFDocumentFileSystemId":null}],"Total":1,"TotalRecords":1,"PageSize":1,"RecordsOnPage":1,"Page":1,"CurrentPage":1,"TotalPages":1}</t>
+          <t>{"Data":[{"Id":16515,"ManifestNumber":null,"DeliveryNumber":0,"RecipientFacilityLicenseNumber":"SF-SBX-NY-6-13402","RecipientFacilityName":"Sandbox AU Distributor","ShipmentTypeName":"Unaffiliated Transfer","ShipmentTransactionType":"Wholesale","InvoiceNumber":"INV-A-0829-1427","PaymentTermDays":null,"PaymentDueDate":null,"EstimatedDepartureDateTime":"2026-08-29T15:28:00.000","ActualDepartureDateTime":null,"EstimatedArrivalDateTime":"2026-08-29T18:28:00.000","ActualArrivalDateTime":null,"GrossWeight":null,"GrossUnitOfWeightId":null,"GrossUnitOfWeightName":null,"PlannedRoute":"Evaluation route.","DeliveryPackageCount":0,"DeliveryReceivedPackageCount":0,"ReceivedDateTime":null,"EstimatedReturnDepartureDateTime":null,"ActualReturnDepartureDateTime":null,"EstimatedReturnArrivalDateTime":null,"ActualReturnArrivalDateTime":null,"RejectedPackagesReturned":false,"PDFDocumentFileSystemId":null}],"Total":1,"TotalRecords":1,"PageSize":1,"RecordsOnPage":1,"Page":1,"CurrentPage":1,"TotalPages":1}</t>
         </is>
       </c>
     </row>
@@ -11452,12 +11452,12 @@
       </c>
       <c r="D21" s="248" t="inlineStr">
         <is>
-          <t>15910</t>
+          <t>16009</t>
         </is>
       </c>
       <c r="E21" s="250" t="inlineStr">
         <is>
-          <t>2026-08-29T13:32:26Z</t>
+          <t>2026-08-29T14:28:07Z</t>
         </is>
       </c>
       <c r="F21" s="247" t="inlineStr">
@@ -11472,7 +11472,7 @@
       </c>
       <c r="H21" s="262" t="inlineStr">
         <is>
-          <t>[{"Name":"TP Template A 0829-1332 (Updated)","TransporterFacilityLicenseNumber":null,"DriverOccupationalLicenseNumber":null,"DriverName":null,"DriverLicenseNumber":null,"PhoneNumberForQuestions":null,"VehicleMake":null,"VehicleModel":null,"VehicleLicensePlateNumber":null,"VehicleRegistrationNumber":null,"Destinations":[{"RecipientLicenseNumber":"SF-SBX-NY-6-13402","InvoiceNumber":"INV-A-0829-1332","TransferTypeName":"Unaffiliated Transfer","PlannedRoute":"Evaluation route.","EstimatedDepartureDateTime":"2026-08-29T14:32:24Z","EstimatedArrivalDateTime":"2026-08-29T17:32:24Z","Transporters":[],"Packages":[],"TransferDestinationId":0}],"TransferTemplateId":15910}]</t>
+          <t>[{"Name":"TP Template A 0829-1427 (Updated)","TransporterFacilityLicenseNumber":null,"DriverOccupationalLicenseNumber":null,"DriverName":null,"DriverLicenseNumber":null,"PhoneNumberForQuestions":null,"VehicleMake":null,"VehicleModel":null,"VehicleLicensePlateNumber":null,"VehicleRegistrationNumber":null,"Destinations":[{"RecipientLicenseNumber":"SF-SBX-NY-6-13402","InvoiceNumber":"INV-A-0829-1427","TransferTypeName":"Unaffiliated Transfer","PlannedRoute":"Evaluation route.","EstimatedDepartureDateTime":"2026-08-29T15:28:06Z","EstimatedArrivalDateTime":"2026-08-29T18:28:06Z","Transporters":[],"Packages":[],"TransferDestinationId":0}],"TransferTemplateId":16009}]</t>
         </is>
       </c>
     </row>
@@ -11853,7 +11853,7 @@
       </c>
       <c r="E5" s="250" t="inlineStr">
         <is>
-          <t>2026-08-29T13:32:26Z</t>
+          <t>2026-08-29T14:28:07Z</t>
         </is>
       </c>
       <c r="F5" s="247" t="inlineStr">
@@ -11868,7 +11868,7 @@
       </c>
       <c r="H5" s="262" t="inlineStr">
         <is>
-          <t>[{"ShipperLicenseNumber":"SF-SBX-NY-6-13402","ShipperName":"Evaluation Shipper","ShipperMainPhoneNumber":"555-000-0000","ShipperAddress1":"1 Evaluation Way","ShipperAddress2":null,"ShipperAddressCity":"Albany","ShipperAddressState":"NY","ShipperAddressPostalCode":"12207","TransporterFacilityLicenseNumber":null,"DriverOccupationalLicenseNumber":null,"DriverName":null,"DriverLicenseNumber":null,"PhoneNumberForQuestions":null,"VehicleMake":null,"VehicleModel":null,"VehicleLicensePlateNumber":null,"VehicleRegistrationNumber":null,"Destinations":[{"RecipientLicenseNumber":"SF-SBX-NY-3-30301","InvoiceNumber":"EXT-A-0829-1332","TransferTypeName":"Beginning Inventory","PlannedRoute":"Evaluation route.","EstimatedDepartureDateTime":"2026-08-29T14:32:26Z","EstimatedArrivalDateTime":"2026-08-29T17:32:26Z","GrossWeight":null,"GrossUnitOfWeightId":null,"Transporters":[],"Packages":[]}]}]</t>
+          <t>[{"ShipperLicenseNumber":"SF-SBX-NY-6-13402","ShipperName":"Evaluation Shipper","ShipperMainPhoneNumber":"555-000-0000","ShipperAddress1":"1 Evaluation Way","ShipperAddress2":null,"ShipperAddressCity":"Albany","ShipperAddressState":"NY","ShipperAddressPostalCode":"12207","TransporterFacilityLicenseNumber":null,"DriverOccupationalLicenseNumber":null,"DriverName":null,"DriverLicenseNumber":null,"PhoneNumberForQuestions":null,"VehicleMake":null,"VehicleModel":null,"VehicleLicensePlateNumber":null,"VehicleRegistrationNumber":null,"Destinations":[{"RecipientLicenseNumber":"SF-SBX-NY-3-30301","InvoiceNumber":"EXT-A-0829-1427","TransferTypeName":"Beginning Inventory","PlannedRoute":"Evaluation route.","EstimatedDepartureDateTime":"2026-08-29T15:28:07Z","EstimatedArrivalDateTime":"2026-08-29T18:28:07Z","GrossWeight":null,"GrossUnitOfWeightId":null,"Transporters":[],"Packages":[]}]}]</t>
         </is>
       </c>
     </row>
@@ -11927,7 +11927,7 @@
       </c>
       <c r="E9" s="250" t="inlineStr">
         <is>
-          <t>2026-08-29T13:32:26Z</t>
+          <t>2026-08-29T14:28:07Z</t>
         </is>
       </c>
       <c r="F9" s="247" t="inlineStr">
@@ -11942,7 +11942,7 @@
       </c>
       <c r="H9" s="262" t="inlineStr">
         <is>
-          <t>[{"ShipperLicenseNumber":"SF-SBX-NY-6-13402","ShipperName":"Evaluation Shipper","ShipperMainPhoneNumber":"555-000-0000","ShipperAddress1":"1 Evaluation Way","ShipperAddress2":null,"ShipperAddressCity":"Albany","ShipperAddressState":"NY","ShipperAddressPostalCode":"12207","TransporterFacilityLicenseNumber":null,"DriverOccupationalLicenseNumber":null,"DriverName":null,"DriverLicenseNumber":null,"PhoneNumberForQuestions":null,"VehicleMake":null,"VehicleModel":null,"VehicleLicensePlateNumber":null,"VehicleRegistrationNumber":null,"Destinations":[{"RecipientLicenseNumber":"SF-SBX-NY-3-30301","InvoiceNumber":"EXT-B-0829-1332","TransferTypeName":"Beginning Inventory","PlannedRoute":"Evaluation route.","EstimatedDepartureDateTime":"2026-08-29T14:32:26Z","EstimatedArrivalDateTime":"2026-08-29T17:32:26Z","GrossWeight":null,"GrossUnitOfWeightId":null,"Transporters":[],"Packages":[]}]}]</t>
+          <t>[{"ShipperLicenseNumber":"SF-SBX-NY-6-13402","ShipperName":"Evaluation Shipper","ShipperMainPhoneNumber":"555-000-0000","ShipperAddress1":"1 Evaluation Way","ShipperAddress2":null,"ShipperAddressCity":"Albany","ShipperAddressState":"NY","ShipperAddressPostalCode":"12207","TransporterFacilityLicenseNumber":null,"DriverOccupationalLicenseNumber":null,"DriverName":null,"DriverLicenseNumber":null,"PhoneNumberForQuestions":null,"VehicleMake":null,"VehicleModel":null,"VehicleLicensePlateNumber":null,"VehicleRegistrationNumber":null,"Destinations":[{"RecipientLicenseNumber":"SF-SBX-NY-3-30301","InvoiceNumber":"EXT-B-0829-1427","TransferTypeName":"Beginning Inventory","PlannedRoute":"Evaluation route.","EstimatedDepartureDateTime":"2026-08-29T15:28:07Z","EstimatedArrivalDateTime":"2026-08-29T18:28:07Z","GrossWeight":null,"GrossUnitOfWeightId":null,"Transporters":[],"Packages":[]}]}]</t>
         </is>
       </c>
     </row>
@@ -12000,7 +12000,7 @@
       </c>
       <c r="E13" s="250" t="inlineStr">
         <is>
-          <t>2026-08-29T13:32:26Z</t>
+          <t>2026-08-29T14:28:07Z</t>
         </is>
       </c>
       <c r="F13" s="247" t="inlineStr">
@@ -12010,7 +12010,7 @@
       </c>
       <c r="G13" s="247" t="inlineStr">
         <is>
-          <t>https://sandbox-api-ny.metrc.com/transfers/v2/incoming?lastModifiedStart=2026-08-28T13%3A32%3A26Z&amp;lastModifiedEnd=2026-08-29T13%3A32%3A26Z&amp;licenseNumber=SF-SBX-NY-3-30301</t>
+          <t>https://sandbox-api-ny.metrc.com/transfers/v2/incoming?lastModifiedStart=2026-08-28T14%3A28%3A07Z&amp;lastModifiedEnd=2026-08-29T14%3A28%3A07Z&amp;licenseNumber=SF-SBX-NY-3-30301</t>
         </is>
       </c>
       <c r="H13" s="262" t="inlineStr">
@@ -15810,12 +15810,12 @@
       </c>
       <c r="D5" s="248" t="inlineStr">
         <is>
-          <t>39528</t>
+          <t>39532</t>
         </is>
       </c>
       <c r="E5" s="250" t="inlineStr">
         <is>
-          <t>Terpenomics Loc 0827-1402</t>
+          <t>Terpenomics Loc 0829-1427</t>
         </is>
       </c>
       <c r="F5" s="247" t="inlineStr">
@@ -15825,7 +15825,7 @@
       </c>
       <c r="G5" s="255" t="inlineStr">
         <is>
-          <t>[{"Name":"Terpenomics Loc 0827-1402","LocationTypeName":"Default Location Type"}]</t>
+          <t>[{"Name":"Terpenomics Loc 0829-1427","LocationTypeName":"Default Location Type"}]</t>
         </is>
       </c>
       <c r="H5" s="247" t="inlineStr">
@@ -15898,12 +15898,12 @@
       </c>
       <c r="D9" s="248" t="inlineStr">
         <is>
-          <t>39528</t>
+          <t>39532</t>
         </is>
       </c>
       <c r="E9" s="250" t="inlineStr">
         <is>
-          <t>Terpenomics Loc 0827-1402 (Updated)</t>
+          <t>Terpenomics Loc 0829-1427 (Updated)</t>
         </is>
       </c>
       <c r="F9" s="247" t="inlineStr">
@@ -15913,7 +15913,7 @@
       </c>
       <c r="G9" s="255" t="inlineStr">
         <is>
-          <t>[{"Id":39528,"Name":"Terpenomics Loc 0827-1402 (Updated)","LocationTypeName":"Default Location Type"}]</t>
+          <t>[{"Id":39532,"Name":"Terpenomics Loc 0829-1427 (Updated)","LocationTypeName":"Default Location Type"}]</t>
         </is>
       </c>
       <c r="H9" s="247" t="inlineStr">
@@ -15978,22 +15978,22 @@
       </c>
       <c r="D13" s="248" t="inlineStr">
         <is>
-          <t>39528</t>
+          <t>39532</t>
         </is>
       </c>
       <c r="E13" s="250" t="inlineStr">
         <is>
-          <t>Terpenomics Loc 0827-1402 (Updated)</t>
+          <t>Terpenomics Loc 0829-1427 (Updated)</t>
         </is>
       </c>
       <c r="F13" s="247" t="inlineStr">
         <is>
-          <t>https://sandbox-api-ny.metrc.com/locations/v2/39528?licenseNumber=SF-SBX-NY-3-30301</t>
+          <t>https://sandbox-api-ny.metrc.com/locations/v2/39532?licenseNumber=SF-SBX-NY-3-30301</t>
         </is>
       </c>
       <c r="G13" s="255" t="inlineStr">
         <is>
-          <t>{"Id":39528,"Name":"Terpenomics Loc 0827-1402 (Updated)","LocationTypeId":1,"LocationTypeName":"Default Location Type","ForPlantBatches":true,"ForPlants":true,"ForHarvests":true,"ForPackages":true}</t>
+          <t>{"Id":39532,"Name":"Terpenomics Loc 0829-1427 (Updated)","LocationTypeId":1,"LocationTypeName":"Default Location Type","ForPlantBatches":true,"ForPlants":true,"ForHarvests":true,"ForPackages":true}</t>
         </is>
       </c>
       <c r="H13" s="247" t="inlineStr">
@@ -16286,12 +16286,12 @@
       </c>
       <c r="D5" s="248" t="inlineStr">
         <is>
-          <t>62112</t>
+          <t>62119</t>
         </is>
       </c>
       <c r="E5" s="250" t="inlineStr">
         <is>
-          <t>Terpenomics Strain 0827-1402</t>
+          <t>Terpenomics Strain 0829-1427</t>
         </is>
       </c>
       <c r="F5" s="247" t="inlineStr">
@@ -16301,7 +16301,7 @@
       </c>
       <c r="G5" s="255" t="inlineStr">
         <is>
-          <t>[{"Name":"Terpenomics Strain 0827-1402","TestingStatus":"None","ThcLevel":0.1865,"CbdLevel":0.1075,"IndicaPercentage":25.0,"SativaPercentage":75.0}]</t>
+          <t>[{"Name":"Terpenomics Strain 0829-1427","TestingStatus":"None","ThcLevel":0.1865,"CbdLevel":0.1075,"IndicaPercentage":25.0,"SativaPercentage":75.0}]</t>
         </is>
       </c>
       <c r="H5" s="247" t="inlineStr">
@@ -16374,12 +16374,12 @@
       </c>
       <c r="D9" s="248" t="inlineStr">
         <is>
-          <t>62112</t>
+          <t>62119</t>
         </is>
       </c>
       <c r="E9" s="250" t="inlineStr">
         <is>
-          <t>Terpenomics Strain 0827-1402</t>
+          <t>Terpenomics Strain 0829-1427</t>
         </is>
       </c>
       <c r="F9" s="247" t="inlineStr">
@@ -16389,7 +16389,7 @@
       </c>
       <c r="G9" s="255" t="inlineStr">
         <is>
-          <t>[{"Id":62112,"Name":"Terpenomics Strain 0827-1402","TestingStatus":"None","ThcLevel":0.1865,"CbdLevel":0.1075,"IndicaPercentage":60.0,"SativaPercentage":40.0}]</t>
+          <t>[{"Id":62119,"Name":"Terpenomics Strain 0829-1427","TestingStatus":"None","ThcLevel":0.1865,"CbdLevel":0.1075,"IndicaPercentage":60.0,"SativaPercentage":40.0}]</t>
         </is>
       </c>
       <c r="H9" s="247" t="inlineStr">
@@ -16454,22 +16454,22 @@
       </c>
       <c r="D13" s="248" t="inlineStr">
         <is>
-          <t>62112</t>
+          <t>62119</t>
         </is>
       </c>
       <c r="E13" s="250" t="inlineStr">
         <is>
-          <t>Terpenomics Strain 0827-1402</t>
+          <t>Terpenomics Strain 0829-1427</t>
         </is>
       </c>
       <c r="F13" s="247" t="inlineStr">
         <is>
-          <t>https://sandbox-api-ny.metrc.com/strains/v2/62112?licenseNumber=SF-SBX-NY-3-30301</t>
+          <t>https://sandbox-api-ny.metrc.com/strains/v2/62119?licenseNumber=SF-SBX-NY-3-30301</t>
         </is>
       </c>
       <c r="G13" s="255" t="inlineStr">
         <is>
-          <t>{"Id":62112,"Name":"Terpenomics Strain 0827-1402","TestingStatus":"None","ThcLevel":0.1865,"CbdLevel":0.1075,"IndicaPercentage":60.0,"SativaPercentage":40.0,"IsUsed":false,"Genetics":"60% Indica / 40% Sativa"}</t>
+          <t>{"Id":62119,"Name":"Terpenomics Strain 0829-1427","TestingStatus":"None","ThcLevel":0.1865,"CbdLevel":0.1075,"IndicaPercentage":60.0,"SativaPercentage":40.0,"IsUsed":false,"Genetics":"60% Indica / 40% Sativa"}</t>
         </is>
       </c>
       <c r="H13" s="247" t="inlineStr">
@@ -16762,12 +16762,12 @@
       </c>
       <c r="D5" s="248" t="inlineStr">
         <is>
-          <t>293817</t>
+          <t>294234</t>
         </is>
       </c>
       <c r="E5" s="250" t="inlineStr">
         <is>
-          <t>Terpenomics Item 0827-1402</t>
+          <t>Terpenomics Item 0829-1427</t>
         </is>
       </c>
       <c r="F5" s="247" t="inlineStr">
@@ -16777,7 +16777,7 @@
       </c>
       <c r="G5" s="255" t="inlineStr">
         <is>
-          <t>[{"ItemCategory":"Bud/Flower - Bulk","Name":"Terpenomics Item 0827-1402","UnitOfMeasure":"Grams","Strain":"Terpenomics Strain 0827-1402"}]</t>
+          <t>[{"ItemCategory":"Bud/Flower - Bulk","Name":"Terpenomics Item 0829-1427","UnitOfMeasure":"Grams","Strain":"Terpenomics Strain 0829-1427"}]</t>
         </is>
       </c>
       <c r="H5" s="247" t="inlineStr">
@@ -16850,12 +16850,12 @@
       </c>
       <c r="D9" s="248" t="inlineStr">
         <is>
-          <t>293817</t>
+          <t>294234</t>
         </is>
       </c>
       <c r="E9" s="250" t="inlineStr">
         <is>
-          <t>Terpenomics Item 0827-1402</t>
+          <t>Terpenomics Item 0829-1427</t>
         </is>
       </c>
       <c r="F9" s="247" t="inlineStr">
@@ -16865,7 +16865,7 @@
       </c>
       <c r="G9" s="255" t="inlineStr">
         <is>
-          <t>[{"ItemCategory":"Bud/Flower - Bulk","Name":"Terpenomics Item 0827-1402","UnitOfMeasure":"Kilograms","Strain":"Terpenomics Strain 0827-1402","Id":293817}]</t>
+          <t>[{"ItemCategory":"Bud/Flower - Bulk","Name":"Terpenomics Item 0829-1427","UnitOfMeasure":"Kilograms","Strain":"Terpenomics Strain 0829-1427","Id":294234}]</t>
         </is>
       </c>
       <c r="H9" s="247" t="inlineStr">
@@ -16930,22 +16930,22 @@
       </c>
       <c r="D13" s="248" t="inlineStr">
         <is>
-          <t>293817</t>
+          <t>294234</t>
         </is>
       </c>
       <c r="E13" s="250" t="inlineStr">
         <is>
-          <t>Terpenomics Item 0827-1402</t>
+          <t>Terpenomics Item 0829-1427</t>
         </is>
       </c>
       <c r="F13" s="247" t="inlineStr">
         <is>
-          <t>https://sandbox-api-ny.metrc.com/items/v2/293817?licenseNumber=SF-SBX-NY-3-30301</t>
+          <t>https://sandbox-api-ny.metrc.com/items/v2/294234?licenseNumber=SF-SBX-NY-3-30301</t>
         </is>
       </c>
       <c r="G13" s="255" t="inlineStr">
         <is>
-          <t>{"Id":293817,"Name":"Terpenomics Item 0827-1402","GlobalProductName":null,"GlobalProductNumber":null,"ProductCategoryName":"Bud/Flower - Bulk","ProductCategoryType":"Buds","IsExpirationDateRequired":false,"HasExpirationDate":false,"IsSellByDateRequired":false,"HasSellByDate":false,"IsUseByDateRequired":false,"HasUseByDate":false,"QuantityType":"WeightBased","DefaultLabTestingState":"NotSubmitted","UnitOfMeasureName":"Kilograms","ApprovalStatus":"Approved","ApprovalStatusDateTime":"2026-08-27T14:02:08+00:00","StrainId":62112,"StrainName":"Terpenomics Strain 0827-1402","ItemBrandId":0,"ItemBrandName":null,"AdministrationMethod":"","UnitCbdPercent":null,"UnitCbdContent":null,"UnitCbdContentUnitOfMeasureName":null,"UnitCbdContentDose":null,"UnitCbdContentDoseUnitOfMeasureName":null,"UnitCbdAPercent":null,"UnitCbdAContent":null,"UnitCbdAContentUnitOfMeasureName":null,"UnitCbdAContentDose":null,"UnitCbdAContentDoseUnitOfMeasureName":null,"UnitThcAPercent":null,"UnitThcAContent":null,"UnitThcAContentUnitOfMeasureName":null,"UnitThcAContentDose":null,"UnitThcAContentDoseUnitOfMeasureId":null,"UnitThcAContentDoseUnitOfMeasureName":null,"UnitThcPercent":null,"UnitThcContent":null,"UnitThcContentUnitOfMeasureName":null,"UnitThcContentDose":null,"UnitThcContentDoseUnitOfMeasureId":null,"UnitThcContentDoseUnitOfMeasureName":null,"UnitVolume":null,"UnitVolumeUnitOfMeasureName":null,"UnitWeight":null,"UnitWeightUnitOfMeasureName":null,"ServingSize":"","NumberOfDoses":null,"UnitQuantity":null,"UnitQuantityUnitOfMeasureName":null,"PublicIngredients":"","Description":"","Allergens":"","ProductImages":[],"ProductPhotoDescription":"","LabelImages":[],"LabelPhotoDescription":"","PackagingImages":[],"PackagingPhotoDescription":"","ProductPDFDocuments":[],"IsUsed":false,"CreatedDateTime":"2026-08-27T14:02:07.54+00:00","LabTestBatchNames":[],"ProcessingJobCategoryName":null,"ProcessingJobTypeName":null,"ProductBrandName":null}</t>
+          <t>{"Id":294234,"Name":"Terpenomics Item 0829-1427","GlobalProductName":null,"GlobalProductNumber":null,"ProductCategoryName":"Bud/Flower - Bulk","ProductCategoryType":"Buds","IsExpirationDateRequired":false,"HasExpirationDate":false,"IsSellByDateRequired":false,"HasSellByDate":false,"IsUseByDateRequired":false,"HasUseByDate":false,"QuantityType":"WeightBased","DefaultLabTestingState":"NotSubmitted","UnitOfMeasureName":"Kilograms","ApprovalStatus":"Approved","ApprovalStatusDateTime":"2026-08-29T14:27:48+00:00","StrainId":62119,"StrainName":"Terpenomics Strain 0829-1427","ItemBrandId":0,"ItemBrandName":null,"AdministrationMethod":"","UnitCbdPercent":null,"UnitCbdContent":null,"UnitCbdContentUnitOfMeasureName":null,"UnitCbdContentDose":null,"UnitCbdContentDoseUnitOfMeasureName":null,"UnitCbdAPercent":null,"UnitCbdAContent":null,"UnitCbdAContentUnitOfMeasureName":null,"UnitCbdAContentDose":null,"UnitCbdAContentDoseUnitOfMeasureName":null,"UnitThcAPercent":null,"UnitThcAContent":null,"UnitThcAContentUnitOfMeasureName":null,"UnitThcAContentDose":null,"UnitThcAContentDoseUnitOfMeasureId":null,"UnitThcAContentDoseUnitOfMeasureName":null,"UnitThcPercent":null,"UnitThcContent":null,"UnitThcContentUnitOfMeasureName":null,"UnitThcContentDose":null,"UnitThcContentDoseUnitOfMeasureId":null,"UnitThcContentDoseUnitOfMeasureName":null,"UnitVolume":null,"UnitVolumeUnitOfMeasureName":null,"UnitWeight":null,"UnitWeightUnitOfMeasureName":null,"ServingSize":"","NumberOfDoses":null,"UnitQuantity":null,"UnitQuantityUnitOfMeasureName":null,"PublicIngredients":"","Description":"","Allergens":"","ProductImages":[],"ProductPhotoDescription":"","LabelImages":[],"LabelPhotoDescription":"","PackagingImages":[],"PackagingPhotoDescription":"","ProductPDFDocuments":[],"IsUsed":false,"CreatedDateTime":"2026-08-29T14:27:47.9+00:00","LabTestBatchNames":[],"ProcessingJobCategoryName":null,"ProcessingJobTypeName":null,"ProductBrandName":null}</t>
         </is>
       </c>
       <c r="H13" s="247" t="inlineStr">

</xml_diff>